<commit_message>
VLED_DCDC_EN 추가, Trim 시퀀스 작성 중
</commit_message>
<xml_diff>
--- a/X-Series/XD12R/Jig/XCR_XDR/XC24RV_XD12RV/Docs/XD12R_TEST_PLAN_260611.xlsx
+++ b/X-Series/XD12R/Jig/XCR_XDR/XC24RV_XD12RV/Docs/XD12R_TEST_PLAN_260611.xlsx
@@ -5,24 +5,25 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sosbi\OneDrive\바탕 화면\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\working\01_Project\FW\X-Series\XD12R\Jig\XCR_XDR\XC24RV_XD12RV\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{645714A8-5C22-448C-98EC-DE6A10D55F30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3205E7ED-3E87-4DDF-B0D1-6D139533BF17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="41020" yWindow="840" windowWidth="34440" windowHeight="19580" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="71880" yWindow="2160" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PIN_PAD" sheetId="3" r:id="rId1"/>
     <sheet name="FT_Test" sheetId="2" r:id="rId2"/>
-    <sheet name="BASIC SETTING" sheetId="4" r:id="rId3"/>
-    <sheet name="SVSYNC INPUT" sheetId="5" r:id="rId4"/>
-    <sheet name="func. test seqeunce" sheetId="6" r:id="rId5"/>
-    <sheet name="PWM_DIV 계산식" sheetId="7" r:id="rId6"/>
-    <sheet name="eFUSE" sheetId="8" r:id="rId7"/>
-    <sheet name="Serial Communication Protocol" sheetId="9" r:id="rId8"/>
-    <sheet name="MIRROR REG. CHECK" sheetId="10" r:id="rId9"/>
-    <sheet name="FUNCTION TEST" sheetId="11" r:id="rId10"/>
+    <sheet name="Sheet1" sheetId="12" r:id="rId3"/>
+    <sheet name="BASIC SETTING" sheetId="4" r:id="rId4"/>
+    <sheet name="SVSYNC INPUT" sheetId="5" r:id="rId5"/>
+    <sheet name="func. test seqeunce" sheetId="6" r:id="rId6"/>
+    <sheet name="PWM_DIV 계산식" sheetId="7" r:id="rId7"/>
+    <sheet name="eFUSE" sheetId="8" r:id="rId8"/>
+    <sheet name="Serial Communication Protocol" sheetId="9" r:id="rId9"/>
+    <sheet name="MIRROR REG. CHECK" sheetId="10" r:id="rId10"/>
+    <sheet name="FUNCTION TEST" sheetId="11" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -1087,7 +1088,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="951" uniqueCount="624">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="954" uniqueCount="628">
   <si>
     <t>Trimming</t>
     <phoneticPr fontId="3" type="noConversion"/>
@@ -4037,292 +4038,6 @@
   <si>
     <t>VERSION1 [11:0]</t>
     <phoneticPr fontId="13" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">CH(N)_EN : 1'd : 1
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">0x05 : 1 / 2 / 4 ….. 200 / 400 / 800
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">TEST EN : 1'd : 1
-SW SEL : 3'd : 1
-PWMOUT_FULL : 1'd : 1
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>0x3F : 830</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-MAX_CURR_LEVEL_(N)[3:0] = 4'd : 3
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>0x19 : FFF , 0x1A : FF</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>---P1---</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-MAX_CURR_VREF_(N)[11:0] = 12'd : (P1)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>0x0A / 0x0B / 0x0C / 0x0D / 0x0E : 12C</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>---P2---</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-MAX_CURR_VREF_(N)[11:0] = 12'd : (P2)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>0x0A / 0x0B / 0x0C / 0x0D / 0x0E : 5DC</t>
-    </r>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">CH(N)_EN : 1'd : 1
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">0x05 : 1 / 2 / 4 ….. 200 / 400 / 800
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">TEST EN : 1'd : 1
-SW SEL : 3'd : 1
-PWMOUT_FULL : 1'd : 1
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>0x3F : 830</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-MAX_CURR_LEVEL_(N)[3:0] = 4'd : 3
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>0x19 : FFF , 0x1A : FF</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>---P3---</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-MAX_CURR_VREF_(N)[11:0] = 12'd : (P3)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>0x0A / 0x0B / 0x0C / 0x0D / 0x0E : C8</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>---P4---</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-MAX_CURR_VREF_(N)[11:0] = 12'd : (P4)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>0x0A / 0x0B / 0x0C / 0x0D / 0x0E : 190</t>
-    </r>
-    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <r>
@@ -4914,9 +4629,441 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>**signed binary**
+    <r>
+      <t xml:space="preserve">**signed binary**
 [2] = signed bit
-[1:0] = data</t>
+[1:0] = data
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF00FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>**signed binary**
+[3] = signed bit
+[2:0] = data</t>
+    </r>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>LDO_DIG</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Sub_Val</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Reg [Table]</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">TEST_EN = 1'd : 1
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF00FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>TEST_ANA_EN[2:0] = 3'd : ????</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+MCLK64_O = 1'd : 1
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>0x3F = 808</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+OSC_MAN_EN = 1'd : 1
+OSC_FLL_MAN [15:0] = 
+16'b : 1000000000000000
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>0x29 : 808</t>
+    </r>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">CH(N)_EN : 1'd : 1
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">0x05 : 1 / 2 / 4 ….. 200 / 400 / 800
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">TEST EN : 1'd : 1
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF00FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>TEST_ANA_EN[2:0] = 3'd : ????</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+SW SEL : 3'd : 1
+PWMOUT_FULL : 1'd : 1
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>0x3F : 830</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+MAX_CURR_LEVEL_(N)[3:0] = 4'd : 3
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">0x19 : FFF , 0x1A : FF
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF00FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>0x19 : 333 , 0x1A : 33??</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>---P1---</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+MAX_CURR_VREF_(N)[11:0] = 12'd : (P1)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>0x0A / 0x0B / 0x0C / 0x0D / 0x0E : 12C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>---P2---</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+MAX_CURR_VREF_(N)[11:0] = 12'd : (P2)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>0x0A / 0x0B / 0x0C / 0x0D / 0x0E : 5DC</t>
+    </r>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">CH(N)_EN : 1'd : 1
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">0x05 : 1 / 2 / 4 ….. 200 / 400 / 800
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">TEST EN : 1'd : 1
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF00FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">TEST_ANA_EN[2:0] = 3'd : ????
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">SW SEL : 3'd : 1
+PWMOUT_FULL : 1'd : 1
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>0x3F : 830</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+MAX_CURR_LEVEL_(N)[3:0] = 4'd : 3
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">0x19 : FFF , 0x1A : FF
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF00FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>0x19 : 333 , 0x1A : 33??</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>---P3---</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+MAX_CURR_VREF_(N)[11:0] = 12'd : (P3)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>0x0A / 0x0B / 0x0C / 0x0D / 0x0E : C8</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>---P4---</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+MAX_CURR_VREF_(N)[11:0] = 12'd : (P4)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>0x0A / 0x0B / 0x0C / 0x0D / 0x0E : 190</t>
+    </r>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -4928,7 +5075,7 @@
     <numFmt numFmtId="176" formatCode="0.000"/>
     <numFmt numFmtId="177" formatCode="0.00000"/>
   </numFmts>
-  <fonts count="34" x14ac:knownFonts="1">
+  <fonts count="36" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -5175,8 +5322,21 @@
       <family val="2"/>
       <charset val="129"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF00FF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF00FF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="18">
+  <fills count="19">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -5279,8 +5439,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="51">
+  <borders count="52">
     <border>
       <left/>
       <right/>
@@ -5916,6 +6082,19 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -5926,7 +6105,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="201">
+  <cellXfs count="214">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -6395,6 +6574,17 @@
     <xf numFmtId="0" fontId="7" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -6440,6 +6630,12 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="48" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="51" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="22" fillId="14" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -6517,6 +6713,12 @@
     </xf>
     <xf numFmtId="0" fontId="22" fillId="16" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="18" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="18" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -6526,6 +6728,11 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFF00FF"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -6832,7 +7039,7 @@
                   <a14:compatExt spid="_x0000_s3073"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-0000010C0000}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0400-0000010C0000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -7006,7 +7213,7 @@
                   <a14:compatExt spid="_x0000_s4098"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0400-000002100000}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0500-000002100000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -7089,15 +7296,15 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>159192</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>6102</xdr:rowOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>648142</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>9277</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>125519</xdr:colOff>
-      <xdr:row>26</xdr:row>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>608119</xdr:colOff>
+      <xdr:row>25</xdr:row>
       <xdr:rowOff>95235</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -7121,8 +7328,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2140392" y="869702"/>
-          <a:ext cx="4589127" cy="4838933"/>
+          <a:off x="648142" y="666502"/>
+          <a:ext cx="4560552" cy="4905608"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -7707,8 +7914,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="660400" y="215900"/>
-          <a:ext cx="8007350" cy="4019550"/>
+          <a:off x="657225" y="219075"/>
+          <a:ext cx="7972425" cy="4076700"/>
           <a:chOff x="645291" y="1818641"/>
           <a:chExt cx="5911073" cy="2754488"/>
         </a:xfrm>
@@ -8655,8 +8862,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="2746375" y="3581400"/>
-          <a:ext cx="3006000" cy="2106000"/>
+          <a:off x="2740025" y="3619500"/>
+          <a:ext cx="3002825" cy="2131400"/>
           <a:chOff x="1864615" y="3049000"/>
           <a:chExt cx="3006000" cy="2106000"/>
         </a:xfrm>
@@ -13636,18 +13843,18 @@
       <c r="O2" s="57"/>
       <c r="P2" s="59"/>
       <c r="Q2" s="54"/>
-      <c r="R2" s="171" t="s">
+      <c r="R2" s="180" t="s">
         <v>94</v>
       </c>
-      <c r="S2" s="171"/>
-      <c r="T2" s="171"/>
-      <c r="U2" s="171"/>
-      <c r="V2" s="171"/>
-      <c r="W2" s="171"/>
-      <c r="X2" s="171"/>
-      <c r="Y2" s="171"/>
-      <c r="Z2" s="171"/>
-      <c r="AA2" s="171"/>
+      <c r="S2" s="180"/>
+      <c r="T2" s="180"/>
+      <c r="U2" s="180"/>
+      <c r="V2" s="180"/>
+      <c r="W2" s="180"/>
+      <c r="X2" s="180"/>
+      <c r="Y2" s="180"/>
+      <c r="Z2" s="180"/>
+      <c r="AA2" s="180"/>
     </row>
     <row r="3" spans="1:27" ht="17.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A3" s="54"/>
@@ -13740,7 +13947,7 @@
       <c r="O4" s="61"/>
       <c r="P4" s="64"/>
       <c r="Q4" s="54"/>
-      <c r="R4" s="172" t="s">
+      <c r="R4" s="181" t="s">
         <v>105</v>
       </c>
       <c r="S4" s="66">
@@ -13781,7 +13988,7 @@
       <c r="O5" s="61"/>
       <c r="P5" s="64"/>
       <c r="Q5" s="54"/>
-      <c r="R5" s="173"/>
+      <c r="R5" s="182"/>
       <c r="S5" s="66">
         <v>2</v>
       </c>
@@ -13828,7 +14035,7 @@
         <v>110</v>
       </c>
       <c r="Q6" s="54"/>
-      <c r="R6" s="173"/>
+      <c r="R6" s="182"/>
       <c r="S6" s="66">
         <v>3</v>
       </c>
@@ -13867,7 +14074,7 @@
       <c r="O7" s="71"/>
       <c r="P7" s="72"/>
       <c r="Q7" s="54"/>
-      <c r="R7" s="173"/>
+      <c r="R7" s="182"/>
       <c r="S7" s="66">
         <v>4</v>
       </c>
@@ -13906,7 +14113,7 @@
       <c r="O8" s="71"/>
       <c r="P8" s="64"/>
       <c r="Q8" s="54"/>
-      <c r="R8" s="173"/>
+      <c r="R8" s="182"/>
       <c r="S8" s="66">
         <v>5</v>
       </c>
@@ -13951,7 +14158,7 @@
       <c r="O9" s="71"/>
       <c r="P9" s="64"/>
       <c r="Q9" s="54"/>
-      <c r="R9" s="174"/>
+      <c r="R9" s="183"/>
       <c r="S9" s="66">
         <v>6</v>
       </c>
@@ -14000,7 +14207,7 @@
         <v>121</v>
       </c>
       <c r="Q10" s="54"/>
-      <c r="R10" s="172" t="s">
+      <c r="R10" s="181" t="s">
         <v>122</v>
       </c>
       <c r="S10" s="66">
@@ -14045,7 +14252,7 @@
         <v>13</v>
       </c>
       <c r="Q11" s="54"/>
-      <c r="R11" s="173"/>
+      <c r="R11" s="182"/>
       <c r="S11" s="66">
         <v>8</v>
       </c>
@@ -14084,7 +14291,7 @@
       <c r="O12" s="71"/>
       <c r="P12" s="64"/>
       <c r="Q12" s="54"/>
-      <c r="R12" s="173"/>
+      <c r="R12" s="182"/>
       <c r="S12" s="66">
         <v>9</v>
       </c>
@@ -14123,7 +14330,7 @@
       <c r="O13" s="71"/>
       <c r="P13" s="64"/>
       <c r="Q13" s="54"/>
-      <c r="R13" s="173"/>
+      <c r="R13" s="182"/>
       <c r="S13" s="66">
         <v>10</v>
       </c>
@@ -14170,7 +14377,7 @@
         <v>121</v>
       </c>
       <c r="Q14" s="54"/>
-      <c r="R14" s="173"/>
+      <c r="R14" s="182"/>
       <c r="S14" s="66">
         <v>11</v>
       </c>
@@ -14211,7 +14418,7 @@
         <v>132</v>
       </c>
       <c r="Q15" s="54"/>
-      <c r="R15" s="174"/>
+      <c r="R15" s="183"/>
       <c r="S15" s="66">
         <v>12</v>
       </c>
@@ -14250,7 +14457,7 @@
       <c r="O16" s="71"/>
       <c r="P16" s="64"/>
       <c r="Q16" s="54"/>
-      <c r="R16" s="172" t="s">
+      <c r="R16" s="181" t="s">
         <v>134</v>
       </c>
       <c r="S16" s="66">
@@ -14297,7 +14504,7 @@
       <c r="O17" s="71"/>
       <c r="P17" s="64"/>
       <c r="Q17" s="54"/>
-      <c r="R17" s="173"/>
+      <c r="R17" s="182"/>
       <c r="S17" s="66">
         <v>14</v>
       </c>
@@ -14350,7 +14557,7 @@
         <v>121</v>
       </c>
       <c r="Q18" s="54"/>
-      <c r="R18" s="173"/>
+      <c r="R18" s="182"/>
       <c r="S18" s="66">
         <v>15</v>
       </c>
@@ -14391,7 +14598,7 @@
         <v>144</v>
       </c>
       <c r="Q19" s="54"/>
-      <c r="R19" s="173"/>
+      <c r="R19" s="182"/>
       <c r="S19" s="66">
         <v>16</v>
       </c>
@@ -14430,7 +14637,7 @@
       <c r="O20" s="71"/>
       <c r="P20" s="64"/>
       <c r="Q20" s="54"/>
-      <c r="R20" s="173"/>
+      <c r="R20" s="182"/>
       <c r="S20" s="66">
         <v>17</v>
       </c>
@@ -14473,7 +14680,7 @@
         <v>147</v>
       </c>
       <c r="Q21" s="54"/>
-      <c r="R21" s="174"/>
+      <c r="R21" s="183"/>
       <c r="S21" s="66">
         <v>18</v>
       </c>
@@ -14520,7 +14727,7 @@
         <v>150</v>
       </c>
       <c r="Q22" s="54"/>
-      <c r="R22" s="172" t="s">
+      <c r="R22" s="181" t="s">
         <v>151</v>
       </c>
       <c r="S22" s="66">
@@ -14561,7 +14768,7 @@
       <c r="O23" s="71"/>
       <c r="P23" s="81"/>
       <c r="Q23" s="54"/>
-      <c r="R23" s="173"/>
+      <c r="R23" s="182"/>
       <c r="S23" s="66">
         <v>20</v>
       </c>
@@ -14600,7 +14807,7 @@
       <c r="O24" s="71"/>
       <c r="P24" s="64"/>
       <c r="Q24" s="54"/>
-      <c r="R24" s="173"/>
+      <c r="R24" s="182"/>
       <c r="S24" s="66">
         <v>21</v>
       </c>
@@ -14639,7 +14846,7 @@
       <c r="O25" s="71"/>
       <c r="P25" s="64"/>
       <c r="Q25" s="54"/>
-      <c r="R25" s="173"/>
+      <c r="R25" s="182"/>
       <c r="S25" s="66">
         <v>22</v>
       </c>
@@ -14686,7 +14893,7 @@
         <v>157</v>
       </c>
       <c r="Q26" s="54"/>
-      <c r="R26" s="173"/>
+      <c r="R26" s="182"/>
       <c r="S26" s="66">
         <v>23</v>
       </c>
@@ -14725,7 +14932,7 @@
       <c r="O27" s="71"/>
       <c r="P27" s="83"/>
       <c r="Q27" s="54"/>
-      <c r="R27" s="174"/>
+      <c r="R27" s="183"/>
       <c r="S27" s="66">
         <v>24</v>
       </c>
@@ -14889,6 +15096,17 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D53A53DC-F305-461A-B42D-7174635AF376}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
+  <sheetData/>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E604ED2C-5422-41B3-894D-0063C8476470}">
   <dimension ref="C3:I11"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
@@ -14901,105 +15119,105 @@
   <sheetData>
     <row r="3" spans="3:9" x14ac:dyDescent="0.45">
       <c r="C3" s="142" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="D3" s="142"/>
       <c r="E3" s="142" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="I3" s="139" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
     </row>
     <row r="4" spans="3:9" x14ac:dyDescent="0.45">
       <c r="C4" s="140" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="D4" s="139" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="E4" s="139" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="I4" s="139" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
     </row>
     <row r="5" spans="3:9" x14ac:dyDescent="0.45">
       <c r="C5" s="140" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="D5" s="139" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
       <c r="E5" s="139" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="I5" s="139" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
     </row>
     <row r="6" spans="3:9" x14ac:dyDescent="0.45">
       <c r="C6" s="140" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="D6" s="139" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="E6" s="139" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="I6" s="139" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
     </row>
     <row r="7" spans="3:9" x14ac:dyDescent="0.45">
       <c r="C7" s="140" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="D7" s="139" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="E7" s="139" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
     </row>
     <row r="8" spans="3:9" x14ac:dyDescent="0.45">
       <c r="C8" s="140" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="D8" s="139" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="E8" s="139" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
     </row>
     <row r="9" spans="3:9" x14ac:dyDescent="0.45">
       <c r="C9" s="140" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
       <c r="D9" s="139"/>
       <c r="E9" s="139" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
     </row>
     <row r="10" spans="3:9" x14ac:dyDescent="0.45">
       <c r="C10" s="140" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
       <c r="D10" s="139"/>
       <c r="E10" s="139" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
     </row>
     <row r="11" spans="3:9" ht="61" x14ac:dyDescent="0.45">
       <c r="C11" s="141" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="D11" s="139"/>
       <c r="E11" s="139" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
     </row>
   </sheetData>
@@ -15034,7 +15252,7 @@
   <sheetData>
     <row r="2" spans="2:13" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="3" spans="2:13" ht="17.5" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B3" s="160" t="s">
+      <c r="B3" s="169" t="s">
         <v>0</v>
       </c>
       <c r="C3" s="1" t="s">
@@ -15072,7 +15290,7 @@
       </c>
     </row>
     <row r="4" spans="2:13" ht="29.5" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B4" s="161"/>
+      <c r="B4" s="170"/>
       <c r="C4" s="22"/>
       <c r="D4" s="89" t="s">
         <v>191</v>
@@ -15090,7 +15308,7 @@
       <c r="M4" s="25"/>
     </row>
     <row r="5" spans="2:13" ht="114" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B5" s="161"/>
+      <c r="B5" s="170"/>
       <c r="C5" s="22" t="s">
         <v>161</v>
       </c>
@@ -15110,7 +15328,7 @@
       <c r="M5" s="25"/>
     </row>
     <row r="6" spans="2:13" ht="43.5" x14ac:dyDescent="0.45">
-      <c r="B6" s="161"/>
+      <c r="B6" s="170"/>
       <c r="C6" s="5">
         <v>1</v>
       </c>
@@ -15143,8 +15361,8 @@
       </c>
       <c r="M6" s="9"/>
     </row>
-    <row r="7" spans="2:13" ht="53" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B7" s="161"/>
+    <row r="7" spans="2:13" ht="101.5" x14ac:dyDescent="0.45">
+      <c r="B7" s="170"/>
       <c r="C7" s="10">
         <v>2</v>
       </c>
@@ -15175,12 +15393,12 @@
       <c r="L7" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="M7" s="14" t="s">
-        <v>623</v>
+      <c r="M7" s="160" t="s">
+        <v>621</v>
       </c>
     </row>
     <row r="8" spans="2:13" ht="43.5" x14ac:dyDescent="0.45">
-      <c r="B8" s="161"/>
+      <c r="B8" s="170"/>
       <c r="C8" s="10">
         <v>3</v>
       </c>
@@ -15206,7 +15424,7 @@
         <v>165</v>
       </c>
       <c r="K8" s="159" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="L8" s="12" t="s">
         <v>22</v>
@@ -15214,7 +15432,7 @@
       <c r="M8" s="14"/>
     </row>
     <row r="9" spans="2:13" ht="43.5" x14ac:dyDescent="0.45">
-      <c r="B9" s="161"/>
+      <c r="B9" s="170"/>
       <c r="C9" s="10">
         <v>4</v>
       </c>
@@ -15247,8 +15465,8 @@
       </c>
       <c r="M9" s="14"/>
     </row>
-    <row r="10" spans="2:13" ht="101.5" x14ac:dyDescent="0.45">
-      <c r="B10" s="161"/>
+    <row r="10" spans="2:13" ht="116" x14ac:dyDescent="0.45">
+      <c r="B10" s="170"/>
       <c r="C10" s="10">
         <v>5</v>
       </c>
@@ -15268,11 +15486,11 @@
       <c r="I10" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="J10" s="13" t="s">
-        <v>171</v>
+      <c r="J10" s="212" t="s">
+        <v>625</v>
       </c>
       <c r="K10" s="159" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="L10" s="12" t="s">
         <v>29</v>
@@ -15282,7 +15500,7 @@
       </c>
     </row>
     <row r="11" spans="2:13" ht="226.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B11" s="161"/>
+      <c r="B11" s="170"/>
       <c r="C11" s="16">
         <v>6</v>
       </c>
@@ -15304,8 +15522,8 @@
       <c r="I11" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="J11" s="18" t="s">
-        <v>566</v>
+      <c r="J11" s="213" t="s">
+        <v>626</v>
       </c>
       <c r="K11" s="18" t="s">
         <v>173</v>
@@ -15318,7 +15536,7 @@
       </c>
     </row>
     <row r="12" spans="2:13" ht="227.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B12" s="161"/>
+      <c r="B12" s="170"/>
       <c r="C12" s="16">
         <v>7</v>
       </c>
@@ -15340,8 +15558,8 @@
       <c r="I12" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="J12" s="18" t="s">
-        <v>567</v>
+      <c r="J12" s="213" t="s">
+        <v>627</v>
       </c>
       <c r="K12" s="18" t="s">
         <v>174</v>
@@ -15350,11 +15568,11 @@
         <v>41</v>
       </c>
       <c r="M12" s="158" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
     </row>
     <row r="13" spans="2:13" ht="63.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B13" s="162"/>
+      <c r="B13" s="171"/>
       <c r="C13" s="47">
         <v>8</v>
       </c>
@@ -15402,7 +15620,7 @@
       <c r="M15" s="21"/>
     </row>
     <row r="16" spans="2:13" ht="17.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B16" s="160" t="s">
+      <c r="B16" s="169" t="s">
         <v>43</v>
       </c>
       <c r="C16" s="22" t="s">
@@ -15440,7 +15658,7 @@
       </c>
     </row>
     <row r="17" spans="2:15" ht="82" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B17" s="163"/>
+      <c r="B17" s="172"/>
       <c r="C17" s="22" t="s">
         <v>161</v>
       </c>
@@ -15460,7 +15678,7 @@
       <c r="M17" s="25"/>
     </row>
     <row r="18" spans="2:15" ht="17.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B18" s="163"/>
+      <c r="B18" s="172"/>
       <c r="C18" s="5">
         <v>1</v>
       </c>
@@ -15486,7 +15704,7 @@
       <c r="M18" s="29"/>
     </row>
     <row r="19" spans="2:15" ht="17.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B19" s="163"/>
+      <c r="B19" s="172"/>
       <c r="C19" s="16">
         <v>2</v>
       </c>
@@ -15514,7 +15732,7 @@
       <c r="M19" s="32"/>
     </row>
     <row r="20" spans="2:15" ht="17.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B20" s="163"/>
+      <c r="B20" s="172"/>
       <c r="C20" s="16">
         <v>3</v>
       </c>
@@ -15540,7 +15758,7 @@
       <c r="M20" s="32"/>
     </row>
     <row r="21" spans="2:15" ht="17.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B21" s="163"/>
+      <c r="B21" s="172"/>
       <c r="C21" s="93">
         <v>4</v>
       </c>
@@ -15566,7 +15784,7 @@
       <c r="M21" s="95"/>
     </row>
     <row r="22" spans="2:15" ht="49.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B22" s="163"/>
+      <c r="B22" s="172"/>
       <c r="C22" s="99"/>
       <c r="D22" s="100" t="s">
         <v>56</v>
@@ -15586,7 +15804,7 @@
       <c r="M22" s="103"/>
     </row>
     <row r="23" spans="2:15" ht="17.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B23" s="163"/>
+      <c r="B23" s="172"/>
       <c r="C23" s="5">
         <v>5</v>
       </c>
@@ -15614,7 +15832,7 @@
       <c r="M23" s="29"/>
     </row>
     <row r="24" spans="2:15" ht="29" x14ac:dyDescent="0.45">
-      <c r="B24" s="163"/>
+      <c r="B24" s="172"/>
       <c r="C24" s="16">
         <v>6</v>
       </c>
@@ -15642,7 +15860,7 @@
       <c r="M24" s="32"/>
     </row>
     <row r="25" spans="2:15" ht="59" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B25" s="163"/>
+      <c r="B25" s="172"/>
       <c r="C25" s="47"/>
       <c r="D25" s="48" t="s">
         <v>188</v>
@@ -15662,7 +15880,7 @@
       <c r="M25" s="91"/>
     </row>
     <row r="26" spans="2:15" ht="59" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B26" s="163"/>
+      <c r="B26" s="172"/>
       <c r="C26" s="10"/>
       <c r="D26" s="104" t="s">
         <v>189</v>
@@ -15682,7 +15900,7 @@
       <c r="M26" s="98"/>
     </row>
     <row r="27" spans="2:15" ht="43.5" x14ac:dyDescent="0.45">
-      <c r="B27" s="163"/>
+      <c r="B27" s="172"/>
       <c r="C27" s="16">
         <v>7</v>
       </c>
@@ -15714,7 +15932,7 @@
       <c r="M27" s="35"/>
     </row>
     <row r="28" spans="2:15" ht="43.5" x14ac:dyDescent="0.45">
-      <c r="B28" s="163"/>
+      <c r="B28" s="172"/>
       <c r="C28" s="16">
         <v>8</v>
       </c>
@@ -15746,7 +15964,7 @@
       <c r="M28" s="35"/>
     </row>
     <row r="29" spans="2:15" ht="43.5" x14ac:dyDescent="0.45">
-      <c r="B29" s="163"/>
+      <c r="B29" s="172"/>
       <c r="C29" s="16">
         <v>9</v>
       </c>
@@ -15778,7 +15996,7 @@
       <c r="M29" s="35"/>
     </row>
     <row r="30" spans="2:15" ht="43.5" x14ac:dyDescent="0.45">
-      <c r="B30" s="163"/>
+      <c r="B30" s="172"/>
       <c r="C30" s="16">
         <v>10</v>
       </c>
@@ -15810,7 +16028,7 @@
       <c r="M30" s="35"/>
     </row>
     <row r="31" spans="2:15" ht="101.5" x14ac:dyDescent="0.45">
-      <c r="B31" s="163"/>
+      <c r="B31" s="172"/>
       <c r="C31" s="16">
         <v>11</v>
       </c>
@@ -15843,7 +16061,7 @@
       <c r="O31" s="108"/>
     </row>
     <row r="32" spans="2:15" ht="197.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B32" s="163"/>
+      <c r="B32" s="172"/>
       <c r="C32" s="16">
         <v>12</v>
       </c>
@@ -15875,7 +16093,7 @@
       <c r="M32" s="32"/>
     </row>
     <row r="33" spans="2:13" ht="291.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B33" s="163"/>
+      <c r="B33" s="172"/>
       <c r="C33" s="16">
         <v>13</v>
       </c>
@@ -15898,7 +16116,7 @@
         <v>35</v>
       </c>
       <c r="J33" s="18" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
       <c r="K33" s="15" t="s">
         <v>70</v>
@@ -15909,7 +16127,7 @@
       <c r="M33" s="37"/>
     </row>
     <row r="34" spans="2:13" ht="409.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B34" s="163"/>
+      <c r="B34" s="172"/>
       <c r="C34" s="16">
         <v>14</v>
       </c>
@@ -15932,7 +16150,7 @@
         <v>35</v>
       </c>
       <c r="J34" s="18" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="K34" s="15" t="s">
         <v>70</v>
@@ -15943,7 +16161,7 @@
       <c r="M34" s="37"/>
     </row>
     <row r="35" spans="2:13" ht="70" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B35" s="163"/>
+      <c r="B35" s="172"/>
       <c r="C35" s="16">
         <v>15</v>
       </c>
@@ -15975,7 +16193,7 @@
       <c r="M35" s="32"/>
     </row>
     <row r="36" spans="2:13" ht="58" x14ac:dyDescent="0.45">
-      <c r="B36" s="163"/>
+      <c r="B36" s="172"/>
       <c r="C36" s="16">
         <v>16</v>
       </c>
@@ -16007,7 +16225,7 @@
       <c r="M36" s="32"/>
     </row>
     <row r="37" spans="2:13" ht="132" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B37" s="163"/>
+      <c r="B37" s="172"/>
       <c r="C37" s="16">
         <v>17</v>
       </c>
@@ -16072,13 +16290,13 @@
     </row>
     <row r="39" spans="2:13" ht="82.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B39" s="148" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="C39" s="99">
         <v>19</v>
       </c>
       <c r="D39" s="107" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="E39" s="100"/>
       <c r="F39" s="149"/>
@@ -16086,7 +16304,7 @@
       <c r="H39" s="150"/>
       <c r="I39" s="151"/>
       <c r="J39" s="153" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="K39" s="100"/>
       <c r="L39" s="107"/>
@@ -16094,13 +16312,13 @@
     </row>
     <row r="40" spans="2:13" ht="57" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B40" s="39" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="C40" s="40">
         <v>20</v>
       </c>
       <c r="D40" s="41" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="E40" s="42"/>
       <c r="F40" s="43" t="s">
@@ -16119,7 +16337,7 @@
       <c r="M40" s="45"/>
     </row>
     <row r="41" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="B41" s="163" t="s">
+      <c r="B41" s="172" t="s">
         <v>90</v>
       </c>
       <c r="C41" s="5">
@@ -16146,12 +16364,12 @@
       <c r="L41" s="28" t="s">
         <v>92</v>
       </c>
-      <c r="M41" s="165" t="s">
-        <v>618</v>
+      <c r="M41" s="174" t="s">
+        <v>616</v>
       </c>
     </row>
     <row r="42" spans="2:13" ht="17" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B42" s="163"/>
+      <c r="B42" s="172"/>
       <c r="C42" s="16">
         <v>22</v>
       </c>
@@ -16176,10 +16394,10 @@
       <c r="L42" s="31" t="s">
         <v>92</v>
       </c>
-      <c r="M42" s="166"/>
+      <c r="M42" s="175"/>
     </row>
     <row r="43" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="B43" s="163"/>
+      <c r="B43" s="172"/>
       <c r="C43" s="16">
         <v>23</v>
       </c>
@@ -16206,10 +16424,10 @@
       <c r="L43" s="31" t="s">
         <v>92</v>
       </c>
-      <c r="M43" s="166"/>
+      <c r="M43" s="175"/>
     </row>
     <row r="44" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="B44" s="163"/>
+      <c r="B44" s="172"/>
       <c r="C44" s="16">
         <v>24</v>
       </c>
@@ -16236,10 +16454,10 @@
       <c r="L44" s="31" t="s">
         <v>92</v>
       </c>
-      <c r="M44" s="166"/>
+      <c r="M44" s="175"/>
     </row>
     <row r="45" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="B45" s="163"/>
+      <c r="B45" s="172"/>
       <c r="C45" s="16">
         <v>25</v>
       </c>
@@ -16268,10 +16486,10 @@
       <c r="L45" s="31" t="s">
         <v>92</v>
       </c>
-      <c r="M45" s="166"/>
+      <c r="M45" s="175"/>
     </row>
     <row r="46" spans="2:13" ht="29" x14ac:dyDescent="0.45">
-      <c r="B46" s="163"/>
+      <c r="B46" s="172"/>
       <c r="C46" s="16">
         <v>26</v>
       </c>
@@ -16298,10 +16516,10 @@
       <c r="L46" s="31" t="s">
         <v>92</v>
       </c>
-      <c r="M46" s="166"/>
+      <c r="M46" s="175"/>
     </row>
     <row r="47" spans="2:13" ht="281" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B47" s="164"/>
+      <c r="B47" s="173"/>
       <c r="C47" s="47">
         <v>27</v>
       </c>
@@ -16324,7 +16542,7 @@
         <v>35</v>
       </c>
       <c r="J47" s="49" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
       <c r="K47" s="49" t="s">
         <v>91</v>
@@ -16332,7 +16550,7 @@
       <c r="L47" s="51" t="s">
         <v>92</v>
       </c>
-      <c r="M47" s="167"/>
+      <c r="M47" s="176"/>
     </row>
     <row r="48" spans="2:13" ht="65" customHeight="1" x14ac:dyDescent="0.45">
       <c r="G48" s="52"/>
@@ -16350,14 +16568,14 @@
       <c r="G52" s="52"/>
     </row>
     <row r="94" spans="3:15" x14ac:dyDescent="0.45">
-      <c r="C94" s="168"/>
-      <c r="D94" s="169"/>
-      <c r="E94" s="169"/>
-      <c r="F94" s="169"/>
-      <c r="G94" s="169"/>
-      <c r="H94" s="169"/>
-      <c r="I94" s="169"/>
-      <c r="J94" s="170"/>
+      <c r="C94" s="177"/>
+      <c r="D94" s="178"/>
+      <c r="E94" s="178"/>
+      <c r="F94" s="178"/>
+      <c r="G94" s="178"/>
+      <c r="H94" s="178"/>
+      <c r="I94" s="178"/>
+      <c r="J94" s="179"/>
       <c r="K94" s="53"/>
       <c r="L94" s="53"/>
       <c r="M94" s="53"/>
@@ -16379,6 +16597,166 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{974E4F1F-3646-43FA-96F3-A95F27E3B023}">
+  <dimension ref="B1:C19"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="3" max="3" width="11.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:3" ht="17.5" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="2" spans="2:3" ht="17.5" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B2" s="184" t="s">
+        <v>622</v>
+      </c>
+      <c r="C2" s="185"/>
+    </row>
+    <row r="3" spans="2:3" ht="17.5" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B3" s="167" t="s">
+        <v>623</v>
+      </c>
+      <c r="C3" s="168" t="s">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B4" s="165">
+        <v>0</v>
+      </c>
+      <c r="C4" s="166">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B5" s="161">
+        <v>1</v>
+      </c>
+      <c r="C5" s="162">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B6" s="161">
+        <v>2</v>
+      </c>
+      <c r="C6" s="162">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B7" s="161">
+        <v>3</v>
+      </c>
+      <c r="C7" s="162">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B8" s="161">
+        <v>4</v>
+      </c>
+      <c r="C8" s="162">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B9" s="161">
+        <v>5</v>
+      </c>
+      <c r="C9" s="162">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B10" s="161">
+        <v>6</v>
+      </c>
+      <c r="C10" s="162">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B11" s="161">
+        <v>7</v>
+      </c>
+      <c r="C11" s="162">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B12" s="161">
+        <v>8</v>
+      </c>
+      <c r="C12" s="162">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B13" s="161">
+        <v>9</v>
+      </c>
+      <c r="C13" s="162">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B14" s="161">
+        <v>10</v>
+      </c>
+      <c r="C14" s="162">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B15" s="161">
+        <v>11</v>
+      </c>
+      <c r="C15" s="162">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B16" s="161">
+        <v>12</v>
+      </c>
+      <c r="C16" s="162">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B17" s="161">
+        <v>13</v>
+      </c>
+      <c r="C17" s="162">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B18" s="161">
+        <v>14</v>
+      </c>
+      <c r="C18" s="162">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3" ht="17.5" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B19" s="163">
+        <v>15</v>
+      </c>
+      <c r="C19" s="164">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:C2"/>
+  </mergeCells>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E2A63BB-3B6E-47AC-A33F-3550900E167A}">
   <dimension ref="B2:S92"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
@@ -16479,13 +16857,13 @@
       <c r="J4" s="117"/>
       <c r="K4" s="118"/>
       <c r="L4" s="118"/>
-      <c r="M4" s="175" t="s">
+      <c r="M4" s="186" t="s">
         <v>220</v>
       </c>
-      <c r="N4" s="175"/>
-      <c r="O4" s="175"/>
-      <c r="P4" s="175"/>
-      <c r="Q4" s="175"/>
+      <c r="N4" s="186"/>
+      <c r="O4" s="186"/>
+      <c r="P4" s="186"/>
+      <c r="Q4" s="186"/>
       <c r="R4" s="109" t="s">
         <v>221</v>
       </c>
@@ -16503,14 +16881,14 @@
       </c>
       <c r="E5" s="115"/>
       <c r="F5" s="117"/>
-      <c r="G5" s="176" t="s">
+      <c r="G5" s="187" t="s">
         <v>225</v>
       </c>
-      <c r="H5" s="177"/>
-      <c r="I5" s="177"/>
-      <c r="J5" s="177"/>
-      <c r="K5" s="177"/>
-      <c r="L5" s="178"/>
+      <c r="H5" s="188"/>
+      <c r="I5" s="188"/>
+      <c r="J5" s="188"/>
+      <c r="K5" s="188"/>
+      <c r="L5" s="189"/>
       <c r="M5" s="116" t="s">
         <v>226</v>
       </c>
@@ -16551,13 +16929,13 @@
       <c r="J6" s="123"/>
       <c r="K6" s="123"/>
       <c r="L6" s="123"/>
-      <c r="M6" s="179" t="s">
+      <c r="M6" s="190" t="s">
         <v>235</v>
       </c>
-      <c r="N6" s="179"/>
-      <c r="O6" s="179"/>
-      <c r="P6" s="179"/>
-      <c r="Q6" s="179"/>
+      <c r="N6" s="190"/>
+      <c r="O6" s="190"/>
+      <c r="P6" s="190"/>
+      <c r="Q6" s="190"/>
       <c r="R6" s="109" t="s">
         <v>236</v>
       </c>
@@ -16576,22 +16954,22 @@
         <v>224</v>
       </c>
       <c r="E7" s="115"/>
-      <c r="F7" s="180" t="s">
+      <c r="F7" s="191" t="s">
         <v>240</v>
       </c>
-      <c r="G7" s="180"/>
-      <c r="H7" s="180"/>
-      <c r="I7" s="180"/>
-      <c r="J7" s="180" t="s">
+      <c r="G7" s="191"/>
+      <c r="H7" s="191"/>
+      <c r="I7" s="191"/>
+      <c r="J7" s="191" t="s">
         <v>241</v>
       </c>
-      <c r="K7" s="180"/>
-      <c r="L7" s="180"/>
-      <c r="M7" s="180"/>
-      <c r="N7" s="180"/>
-      <c r="O7" s="180"/>
-      <c r="P7" s="180"/>
-      <c r="Q7" s="180"/>
+      <c r="K7" s="191"/>
+      <c r="L7" s="191"/>
+      <c r="M7" s="191"/>
+      <c r="N7" s="191"/>
+      <c r="O7" s="191"/>
+      <c r="P7" s="191"/>
+      <c r="Q7" s="191"/>
       <c r="R7" s="109" t="s">
         <v>242</v>
       </c>
@@ -16610,22 +16988,22 @@
         <v>224</v>
       </c>
       <c r="E8" s="115"/>
-      <c r="F8" s="180" t="s">
+      <c r="F8" s="191" t="s">
         <v>246</v>
       </c>
-      <c r="G8" s="180"/>
-      <c r="H8" s="180"/>
-      <c r="I8" s="180"/>
-      <c r="J8" s="180"/>
-      <c r="K8" s="180"/>
-      <c r="L8" s="180"/>
-      <c r="M8" s="180"/>
-      <c r="N8" s="180" t="s">
+      <c r="G8" s="191"/>
+      <c r="H8" s="191"/>
+      <c r="I8" s="191"/>
+      <c r="J8" s="191"/>
+      <c r="K8" s="191"/>
+      <c r="L8" s="191"/>
+      <c r="M8" s="191"/>
+      <c r="N8" s="191" t="s">
         <v>247</v>
       </c>
-      <c r="O8" s="180"/>
-      <c r="P8" s="180"/>
-      <c r="Q8" s="180"/>
+      <c r="O8" s="191"/>
+      <c r="P8" s="191"/>
+      <c r="Q8" s="191"/>
       <c r="S8" s="113" t="s">
         <v>248</v>
       </c>
@@ -16695,16 +17073,16 @@
         <v>224</v>
       </c>
       <c r="E10" s="115"/>
-      <c r="F10" s="183" t="s">
+      <c r="F10" s="194" t="s">
         <v>267</v>
       </c>
-      <c r="G10" s="184"/>
-      <c r="H10" s="185" t="s">
+      <c r="G10" s="195"/>
+      <c r="H10" s="196" t="s">
         <v>268</v>
       </c>
-      <c r="I10" s="186"/>
-      <c r="J10" s="186"/>
-      <c r="K10" s="184"/>
+      <c r="I10" s="197"/>
+      <c r="J10" s="197"/>
+      <c r="K10" s="195"/>
       <c r="L10" s="116" t="s">
         <v>269</v>
       </c>
@@ -16741,30 +17119,30 @@
         <v>279</v>
       </c>
       <c r="E11" s="115"/>
-      <c r="F11" s="181" t="s">
+      <c r="F11" s="192" t="s">
         <v>280</v>
       </c>
-      <c r="G11" s="182"/>
-      <c r="H11" s="181" t="s">
+      <c r="G11" s="193"/>
+      <c r="H11" s="192" t="s">
         <v>281</v>
       </c>
-      <c r="I11" s="182"/>
-      <c r="J11" s="181" t="s">
+      <c r="I11" s="193"/>
+      <c r="J11" s="192" t="s">
         <v>282</v>
       </c>
-      <c r="K11" s="182"/>
-      <c r="L11" s="181" t="s">
+      <c r="K11" s="193"/>
+      <c r="L11" s="192" t="s">
         <v>283</v>
       </c>
-      <c r="M11" s="182"/>
-      <c r="N11" s="181" t="s">
+      <c r="M11" s="193"/>
+      <c r="N11" s="192" t="s">
         <v>284</v>
       </c>
-      <c r="O11" s="182"/>
-      <c r="P11" s="181" t="s">
+      <c r="O11" s="193"/>
+      <c r="P11" s="192" t="s">
         <v>285</v>
       </c>
-      <c r="Q11" s="182"/>
+      <c r="Q11" s="193"/>
       <c r="R11" s="109" t="s">
         <v>286</v>
       </c>
@@ -16783,30 +17161,30 @@
         <v>279</v>
       </c>
       <c r="E12" s="115"/>
-      <c r="F12" s="181" t="s">
+      <c r="F12" s="192" t="s">
         <v>290</v>
       </c>
-      <c r="G12" s="182"/>
-      <c r="H12" s="181" t="s">
+      <c r="G12" s="193"/>
+      <c r="H12" s="192" t="s">
         <v>291</v>
       </c>
-      <c r="I12" s="182"/>
-      <c r="J12" s="181" t="s">
+      <c r="I12" s="193"/>
+      <c r="J12" s="192" t="s">
         <v>292</v>
       </c>
-      <c r="K12" s="182"/>
-      <c r="L12" s="181" t="s">
+      <c r="K12" s="193"/>
+      <c r="L12" s="192" t="s">
         <v>293</v>
       </c>
-      <c r="M12" s="182"/>
-      <c r="N12" s="181" t="s">
+      <c r="M12" s="193"/>
+      <c r="N12" s="192" t="s">
         <v>294</v>
       </c>
-      <c r="O12" s="182"/>
-      <c r="P12" s="181" t="s">
+      <c r="O12" s="193"/>
+      <c r="P12" s="192" t="s">
         <v>295</v>
       </c>
-      <c r="Q12" s="182"/>
+      <c r="Q12" s="193"/>
       <c r="S12" s="113" t="s">
         <v>287</v>
       </c>
@@ -16890,20 +17268,20 @@
         <v>279</v>
       </c>
       <c r="E15" s="115"/>
-      <c r="F15" s="187" t="s">
+      <c r="F15" s="198" t="s">
         <v>312</v>
       </c>
-      <c r="G15" s="188"/>
-      <c r="H15" s="188"/>
-      <c r="I15" s="188"/>
-      <c r="J15" s="188"/>
-      <c r="K15" s="188"/>
-      <c r="L15" s="188"/>
-      <c r="M15" s="188"/>
-      <c r="N15" s="188"/>
-      <c r="O15" s="188"/>
-      <c r="P15" s="188"/>
-      <c r="Q15" s="182"/>
+      <c r="G15" s="199"/>
+      <c r="H15" s="199"/>
+      <c r="I15" s="199"/>
+      <c r="J15" s="199"/>
+      <c r="K15" s="199"/>
+      <c r="L15" s="199"/>
+      <c r="M15" s="199"/>
+      <c r="N15" s="199"/>
+      <c r="O15" s="199"/>
+      <c r="P15" s="199"/>
+      <c r="Q15" s="193"/>
       <c r="R15" s="109" t="s">
         <v>313</v>
       </c>
@@ -16922,20 +17300,20 @@
         <v>279</v>
       </c>
       <c r="E16" s="115"/>
-      <c r="F16" s="187" t="s">
+      <c r="F16" s="198" t="s">
         <v>317</v>
       </c>
-      <c r="G16" s="188"/>
-      <c r="H16" s="188"/>
-      <c r="I16" s="188"/>
-      <c r="J16" s="188"/>
-      <c r="K16" s="188"/>
-      <c r="L16" s="188"/>
-      <c r="M16" s="188"/>
-      <c r="N16" s="188"/>
-      <c r="O16" s="188"/>
-      <c r="P16" s="188"/>
-      <c r="Q16" s="182"/>
+      <c r="G16" s="199"/>
+      <c r="H16" s="199"/>
+      <c r="I16" s="199"/>
+      <c r="J16" s="199"/>
+      <c r="K16" s="199"/>
+      <c r="L16" s="199"/>
+      <c r="M16" s="199"/>
+      <c r="N16" s="199"/>
+      <c r="O16" s="199"/>
+      <c r="P16" s="199"/>
+      <c r="Q16" s="193"/>
       <c r="R16" s="109" t="s">
         <v>318</v>
       </c>
@@ -16954,20 +17332,20 @@
         <v>279</v>
       </c>
       <c r="E17" s="115"/>
-      <c r="F17" s="175" t="s">
+      <c r="F17" s="186" t="s">
         <v>321</v>
       </c>
-      <c r="G17" s="175"/>
-      <c r="H17" s="175"/>
-      <c r="I17" s="175"/>
-      <c r="J17" s="175"/>
-      <c r="K17" s="175"/>
-      <c r="L17" s="175"/>
-      <c r="M17" s="175"/>
-      <c r="N17" s="175"/>
-      <c r="O17" s="175"/>
-      <c r="P17" s="175"/>
-      <c r="Q17" s="175"/>
+      <c r="G17" s="186"/>
+      <c r="H17" s="186"/>
+      <c r="I17" s="186"/>
+      <c r="J17" s="186"/>
+      <c r="K17" s="186"/>
+      <c r="L17" s="186"/>
+      <c r="M17" s="186"/>
+      <c r="N17" s="186"/>
+      <c r="O17" s="186"/>
+      <c r="P17" s="186"/>
+      <c r="Q17" s="186"/>
       <c r="R17" s="109" t="s">
         <v>322</v>
       </c>
@@ -16986,20 +17364,20 @@
         <v>279</v>
       </c>
       <c r="E18" s="115"/>
-      <c r="F18" s="175" t="s">
+      <c r="F18" s="186" t="s">
         <v>325</v>
       </c>
-      <c r="G18" s="175"/>
-      <c r="H18" s="175"/>
-      <c r="I18" s="175"/>
-      <c r="J18" s="175"/>
-      <c r="K18" s="175"/>
-      <c r="L18" s="175"/>
-      <c r="M18" s="175"/>
-      <c r="N18" s="175"/>
-      <c r="O18" s="175"/>
-      <c r="P18" s="175"/>
-      <c r="Q18" s="175"/>
+      <c r="G18" s="186"/>
+      <c r="H18" s="186"/>
+      <c r="I18" s="186"/>
+      <c r="J18" s="186"/>
+      <c r="K18" s="186"/>
+      <c r="L18" s="186"/>
+      <c r="M18" s="186"/>
+      <c r="N18" s="186"/>
+      <c r="O18" s="186"/>
+      <c r="P18" s="186"/>
+      <c r="Q18" s="186"/>
       <c r="S18" s="113" t="s">
         <v>326</v>
       </c>
@@ -17015,20 +17393,20 @@
         <v>279</v>
       </c>
       <c r="E19" s="115"/>
-      <c r="F19" s="175" t="s">
+      <c r="F19" s="186" t="s">
         <v>329</v>
       </c>
-      <c r="G19" s="175"/>
-      <c r="H19" s="175"/>
-      <c r="I19" s="175"/>
-      <c r="J19" s="175"/>
-      <c r="K19" s="175"/>
-      <c r="L19" s="175"/>
-      <c r="M19" s="175"/>
-      <c r="N19" s="175"/>
-      <c r="O19" s="175"/>
-      <c r="P19" s="175"/>
-      <c r="Q19" s="175"/>
+      <c r="G19" s="186"/>
+      <c r="H19" s="186"/>
+      <c r="I19" s="186"/>
+      <c r="J19" s="186"/>
+      <c r="K19" s="186"/>
+      <c r="L19" s="186"/>
+      <c r="M19" s="186"/>
+      <c r="N19" s="186"/>
+      <c r="O19" s="186"/>
+      <c r="P19" s="186"/>
+      <c r="Q19" s="186"/>
       <c r="S19" s="113" t="s">
         <v>326</v>
       </c>
@@ -17069,20 +17447,20 @@
       <c r="E21" s="115"/>
       <c r="F21" s="125"/>
       <c r="G21" s="125"/>
-      <c r="H21" s="180" t="s">
+      <c r="H21" s="191" t="s">
         <v>334</v>
       </c>
-      <c r="I21" s="180"/>
-      <c r="J21" s="180"/>
-      <c r="K21" s="180"/>
-      <c r="L21" s="180"/>
-      <c r="M21" s="180" t="s">
+      <c r="I21" s="191"/>
+      <c r="J21" s="191"/>
+      <c r="K21" s="191"/>
+      <c r="L21" s="191"/>
+      <c r="M21" s="191" t="s">
         <v>335</v>
       </c>
-      <c r="N21" s="180"/>
-      <c r="O21" s="180"/>
-      <c r="P21" s="180"/>
-      <c r="Q21" s="180"/>
+      <c r="N21" s="191"/>
+      <c r="O21" s="191"/>
+      <c r="P21" s="191"/>
+      <c r="Q21" s="191"/>
       <c r="R21" s="109" t="s">
         <v>336</v>
       </c>
@@ -17103,20 +17481,20 @@
       <c r="E22" s="115"/>
       <c r="F22" s="125"/>
       <c r="G22" s="125"/>
-      <c r="H22" s="180" t="s">
+      <c r="H22" s="191" t="s">
         <v>340</v>
       </c>
-      <c r="I22" s="180"/>
-      <c r="J22" s="180"/>
-      <c r="K22" s="180"/>
-      <c r="L22" s="180"/>
-      <c r="M22" s="180" t="s">
+      <c r="I22" s="191"/>
+      <c r="J22" s="191"/>
+      <c r="K22" s="191"/>
+      <c r="L22" s="191"/>
+      <c r="M22" s="191" t="s">
         <v>341</v>
       </c>
-      <c r="N22" s="180"/>
-      <c r="O22" s="180"/>
-      <c r="P22" s="180"/>
-      <c r="Q22" s="180"/>
+      <c r="N22" s="191"/>
+      <c r="O22" s="191"/>
+      <c r="P22" s="191"/>
+      <c r="Q22" s="191"/>
       <c r="S22" s="113" t="s">
         <v>342</v>
       </c>
@@ -17134,20 +17512,20 @@
       <c r="E23" s="115"/>
       <c r="F23" s="125"/>
       <c r="G23" s="125"/>
-      <c r="H23" s="180" t="s">
+      <c r="H23" s="191" t="s">
         <v>345</v>
       </c>
-      <c r="I23" s="180"/>
-      <c r="J23" s="180"/>
-      <c r="K23" s="180"/>
-      <c r="L23" s="180"/>
-      <c r="M23" s="180" t="s">
+      <c r="I23" s="191"/>
+      <c r="J23" s="191"/>
+      <c r="K23" s="191"/>
+      <c r="L23" s="191"/>
+      <c r="M23" s="191" t="s">
         <v>346</v>
       </c>
-      <c r="N23" s="180"/>
-      <c r="O23" s="180"/>
-      <c r="P23" s="180"/>
-      <c r="Q23" s="180"/>
+      <c r="N23" s="191"/>
+      <c r="O23" s="191"/>
+      <c r="P23" s="191"/>
+      <c r="Q23" s="191"/>
       <c r="S23" s="113" t="s">
         <v>347</v>
       </c>
@@ -17165,20 +17543,20 @@
       <c r="E24" s="115"/>
       <c r="F24" s="125"/>
       <c r="G24" s="125"/>
-      <c r="H24" s="180" t="s">
+      <c r="H24" s="191" t="s">
         <v>350</v>
       </c>
-      <c r="I24" s="180"/>
-      <c r="J24" s="180"/>
-      <c r="K24" s="180"/>
-      <c r="L24" s="180"/>
-      <c r="M24" s="180" t="s">
+      <c r="I24" s="191"/>
+      <c r="J24" s="191"/>
+      <c r="K24" s="191"/>
+      <c r="L24" s="191"/>
+      <c r="M24" s="191" t="s">
         <v>351</v>
       </c>
-      <c r="N24" s="180"/>
-      <c r="O24" s="180"/>
-      <c r="P24" s="180"/>
-      <c r="Q24" s="180"/>
+      <c r="N24" s="191"/>
+      <c r="O24" s="191"/>
+      <c r="P24" s="191"/>
+      <c r="Q24" s="191"/>
       <c r="S24" s="113" t="s">
         <v>352</v>
       </c>
@@ -17196,20 +17574,20 @@
       <c r="E25" s="115"/>
       <c r="F25" s="125"/>
       <c r="G25" s="125"/>
-      <c r="H25" s="180" t="s">
+      <c r="H25" s="191" t="s">
         <v>355</v>
       </c>
-      <c r="I25" s="180"/>
-      <c r="J25" s="180"/>
-      <c r="K25" s="180"/>
-      <c r="L25" s="180"/>
-      <c r="M25" s="180" t="s">
+      <c r="I25" s="191"/>
+      <c r="J25" s="191"/>
+      <c r="K25" s="191"/>
+      <c r="L25" s="191"/>
+      <c r="M25" s="191" t="s">
         <v>356</v>
       </c>
-      <c r="N25" s="180"/>
-      <c r="O25" s="180"/>
-      <c r="P25" s="180"/>
-      <c r="Q25" s="180"/>
+      <c r="N25" s="191"/>
+      <c r="O25" s="191"/>
+      <c r="P25" s="191"/>
+      <c r="Q25" s="191"/>
       <c r="S25" s="113" t="s">
         <v>357</v>
       </c>
@@ -17227,20 +17605,20 @@
       <c r="E26" s="115"/>
       <c r="F26" s="125"/>
       <c r="G26" s="125"/>
-      <c r="H26" s="180" t="s">
+      <c r="H26" s="191" t="s">
         <v>360</v>
       </c>
-      <c r="I26" s="180"/>
-      <c r="J26" s="180"/>
-      <c r="K26" s="180"/>
-      <c r="L26" s="180"/>
-      <c r="M26" s="180" t="s">
+      <c r="I26" s="191"/>
+      <c r="J26" s="191"/>
+      <c r="K26" s="191"/>
+      <c r="L26" s="191"/>
+      <c r="M26" s="191" t="s">
         <v>361</v>
       </c>
-      <c r="N26" s="180"/>
-      <c r="O26" s="180"/>
-      <c r="P26" s="180"/>
-      <c r="Q26" s="180"/>
+      <c r="N26" s="191"/>
+      <c r="O26" s="191"/>
+      <c r="P26" s="191"/>
+      <c r="Q26" s="191"/>
       <c r="S26" s="113" t="s">
         <v>362</v>
       </c>
@@ -17256,26 +17634,26 @@
         <v>224</v>
       </c>
       <c r="E27" s="115"/>
-      <c r="F27" s="189" t="s">
+      <c r="F27" s="200" t="s">
         <v>365</v>
       </c>
-      <c r="G27" s="189"/>
-      <c r="H27" s="189"/>
-      <c r="I27" s="189" t="s">
+      <c r="G27" s="200"/>
+      <c r="H27" s="200"/>
+      <c r="I27" s="200" t="s">
         <v>366</v>
       </c>
-      <c r="J27" s="189"/>
-      <c r="K27" s="189"/>
-      <c r="L27" s="189" t="s">
+      <c r="J27" s="200"/>
+      <c r="K27" s="200"/>
+      <c r="L27" s="200" t="s">
         <v>367</v>
       </c>
-      <c r="M27" s="189"/>
-      <c r="N27" s="189"/>
-      <c r="O27" s="189" t="s">
+      <c r="M27" s="200"/>
+      <c r="N27" s="200"/>
+      <c r="O27" s="200" t="s">
         <v>368</v>
       </c>
-      <c r="P27" s="189"/>
-      <c r="Q27" s="189"/>
+      <c r="P27" s="200"/>
+      <c r="Q27" s="200"/>
       <c r="R27" s="109" t="s">
         <v>369</v>
       </c>
@@ -17294,26 +17672,26 @@
         <v>224</v>
       </c>
       <c r="E28" s="115"/>
-      <c r="F28" s="189" t="s">
+      <c r="F28" s="200" t="s">
         <v>372</v>
       </c>
-      <c r="G28" s="189"/>
-      <c r="H28" s="189"/>
-      <c r="I28" s="190" t="s">
+      <c r="G28" s="200"/>
+      <c r="H28" s="200"/>
+      <c r="I28" s="201" t="s">
         <v>373</v>
       </c>
-      <c r="J28" s="191"/>
-      <c r="K28" s="192"/>
-      <c r="L28" s="189" t="s">
+      <c r="J28" s="202"/>
+      <c r="K28" s="203"/>
+      <c r="L28" s="200" t="s">
         <v>374</v>
       </c>
-      <c r="M28" s="189"/>
-      <c r="N28" s="189"/>
-      <c r="O28" s="189" t="s">
+      <c r="M28" s="200"/>
+      <c r="N28" s="200"/>
+      <c r="O28" s="200" t="s">
         <v>375</v>
       </c>
-      <c r="P28" s="189"/>
-      <c r="Q28" s="189"/>
+      <c r="P28" s="200"/>
+      <c r="Q28" s="200"/>
       <c r="S28" s="113" t="s">
         <v>376</v>
       </c>
@@ -17335,16 +17713,16 @@
       <c r="I29" s="117"/>
       <c r="J29" s="117"/>
       <c r="K29" s="117"/>
-      <c r="L29" s="189" t="s">
+      <c r="L29" s="200" t="s">
         <v>379</v>
       </c>
-      <c r="M29" s="189"/>
-      <c r="N29" s="189"/>
-      <c r="O29" s="189" t="s">
+      <c r="M29" s="200"/>
+      <c r="N29" s="200"/>
+      <c r="O29" s="200" t="s">
         <v>380</v>
       </c>
-      <c r="P29" s="189"/>
-      <c r="Q29" s="189"/>
+      <c r="P29" s="200"/>
+      <c r="Q29" s="200"/>
       <c r="S29" s="113" t="s">
         <v>381</v>
       </c>
@@ -17360,24 +17738,24 @@
         <v>279</v>
       </c>
       <c r="E30" s="115"/>
-      <c r="F30" s="193" t="s">
+      <c r="F30" s="204" t="s">
         <v>384</v>
       </c>
-      <c r="G30" s="193"/>
-      <c r="H30" s="193"/>
-      <c r="I30" s="193"/>
-      <c r="J30" s="193" t="s">
+      <c r="G30" s="204"/>
+      <c r="H30" s="204"/>
+      <c r="I30" s="204"/>
+      <c r="J30" s="204" t="s">
         <v>385</v>
       </c>
-      <c r="K30" s="193"/>
-      <c r="L30" s="193"/>
-      <c r="M30" s="193"/>
-      <c r="N30" s="193" t="s">
+      <c r="K30" s="204"/>
+      <c r="L30" s="204"/>
+      <c r="M30" s="204"/>
+      <c r="N30" s="204" t="s">
         <v>386</v>
       </c>
-      <c r="O30" s="193"/>
-      <c r="P30" s="193"/>
-      <c r="Q30" s="193"/>
+      <c r="O30" s="204"/>
+      <c r="P30" s="204"/>
+      <c r="Q30" s="204"/>
       <c r="R30" s="109" t="s">
         <v>387</v>
       </c>
@@ -17400,18 +17778,18 @@
       <c r="G31" s="117"/>
       <c r="H31" s="117"/>
       <c r="I31" s="117"/>
-      <c r="J31" s="193" t="s">
+      <c r="J31" s="204" t="s">
         <v>391</v>
       </c>
-      <c r="K31" s="193"/>
-      <c r="L31" s="193"/>
-      <c r="M31" s="193"/>
-      <c r="N31" s="193" t="s">
+      <c r="K31" s="204"/>
+      <c r="L31" s="204"/>
+      <c r="M31" s="204"/>
+      <c r="N31" s="204" t="s">
         <v>392</v>
       </c>
-      <c r="O31" s="193"/>
-      <c r="P31" s="193"/>
-      <c r="Q31" s="193"/>
+      <c r="O31" s="204"/>
+      <c r="P31" s="204"/>
+      <c r="Q31" s="204"/>
       <c r="S31" s="113" t="s">
         <v>326</v>
       </c>
@@ -17459,22 +17837,22 @@
         <v>400</v>
       </c>
       <c r="E33" s="115"/>
-      <c r="F33" s="180" t="s">
+      <c r="F33" s="191" t="s">
         <v>401</v>
       </c>
-      <c r="G33" s="180"/>
-      <c r="H33" s="180"/>
-      <c r="I33" s="180"/>
-      <c r="J33" s="180"/>
-      <c r="K33" s="180"/>
-      <c r="L33" s="180" t="s">
+      <c r="G33" s="191"/>
+      <c r="H33" s="191"/>
+      <c r="I33" s="191"/>
+      <c r="J33" s="191"/>
+      <c r="K33" s="191"/>
+      <c r="L33" s="191" t="s">
         <v>402</v>
       </c>
-      <c r="M33" s="180"/>
-      <c r="N33" s="180"/>
-      <c r="O33" s="180"/>
-      <c r="P33" s="180"/>
-      <c r="Q33" s="180"/>
+      <c r="M33" s="191"/>
+      <c r="N33" s="191"/>
+      <c r="O33" s="191"/>
+      <c r="P33" s="191"/>
+      <c r="Q33" s="191"/>
       <c r="R33" s="109" t="s">
         <v>221</v>
       </c>
@@ -17494,17 +17872,17 @@
       <c r="F34" s="117"/>
       <c r="G34" s="117"/>
       <c r="H34" s="117"/>
-      <c r="I34" s="180" t="s">
+      <c r="I34" s="191" t="s">
         <v>406</v>
       </c>
-      <c r="J34" s="180"/>
-      <c r="K34" s="180"/>
-      <c r="L34" s="180"/>
-      <c r="M34" s="180"/>
-      <c r="N34" s="180"/>
-      <c r="O34" s="180"/>
-      <c r="P34" s="180"/>
-      <c r="Q34" s="180"/>
+      <c r="J34" s="191"/>
+      <c r="K34" s="191"/>
+      <c r="L34" s="191"/>
+      <c r="M34" s="191"/>
+      <c r="N34" s="191"/>
+      <c r="O34" s="191"/>
+      <c r="P34" s="191"/>
+      <c r="Q34" s="191"/>
       <c r="R34" s="109" t="s">
         <v>221</v>
       </c>
@@ -17523,18 +17901,18 @@
       <c r="E35" s="115"/>
       <c r="F35" s="117"/>
       <c r="G35" s="117"/>
-      <c r="H35" s="180" t="s">
+      <c r="H35" s="191" t="s">
         <v>409</v>
       </c>
-      <c r="I35" s="180"/>
-      <c r="J35" s="180"/>
-      <c r="K35" s="180"/>
-      <c r="L35" s="180"/>
-      <c r="M35" s="180"/>
-      <c r="N35" s="180"/>
-      <c r="O35" s="180"/>
-      <c r="P35" s="180"/>
-      <c r="Q35" s="180"/>
+      <c r="I35" s="191"/>
+      <c r="J35" s="191"/>
+      <c r="K35" s="191"/>
+      <c r="L35" s="191"/>
+      <c r="M35" s="191"/>
+      <c r="N35" s="191"/>
+      <c r="O35" s="191"/>
+      <c r="P35" s="191"/>
+      <c r="Q35" s="191"/>
       <c r="R35" s="109" t="s">
         <v>221</v>
       </c>
@@ -17555,18 +17933,18 @@
         <v>412</v>
       </c>
       <c r="G36" s="117"/>
-      <c r="H36" s="180" t="s">
+      <c r="H36" s="191" t="s">
         <v>413</v>
       </c>
-      <c r="I36" s="180"/>
-      <c r="J36" s="180"/>
-      <c r="K36" s="180"/>
-      <c r="L36" s="180"/>
-      <c r="M36" s="180"/>
-      <c r="N36" s="180"/>
-      <c r="O36" s="180"/>
-      <c r="P36" s="180"/>
-      <c r="Q36" s="180"/>
+      <c r="I36" s="191"/>
+      <c r="J36" s="191"/>
+      <c r="K36" s="191"/>
+      <c r="L36" s="191"/>
+      <c r="M36" s="191"/>
+      <c r="N36" s="191"/>
+      <c r="O36" s="191"/>
+      <c r="P36" s="191"/>
+      <c r="Q36" s="191"/>
       <c r="R36" s="109" t="s">
         <v>414</v>
       </c>
@@ -17585,18 +17963,18 @@
       <c r="E37" s="115"/>
       <c r="F37" s="125"/>
       <c r="G37" s="125"/>
-      <c r="H37" s="180" t="s">
+      <c r="H37" s="191" t="s">
         <v>417</v>
       </c>
-      <c r="I37" s="180"/>
-      <c r="J37" s="180"/>
-      <c r="K37" s="180"/>
-      <c r="L37" s="180"/>
-      <c r="M37" s="180"/>
-      <c r="N37" s="180"/>
-      <c r="O37" s="180"/>
-      <c r="P37" s="180"/>
-      <c r="Q37" s="180"/>
+      <c r="I37" s="191"/>
+      <c r="J37" s="191"/>
+      <c r="K37" s="191"/>
+      <c r="L37" s="191"/>
+      <c r="M37" s="191"/>
+      <c r="N37" s="191"/>
+      <c r="O37" s="191"/>
+      <c r="P37" s="191"/>
+      <c r="Q37" s="191"/>
       <c r="R37" s="109" t="s">
         <v>221</v>
       </c>
@@ -17614,19 +17992,19 @@
       </c>
       <c r="E38" s="115"/>
       <c r="F38" s="125"/>
-      <c r="G38" s="180" t="s">
+      <c r="G38" s="191" t="s">
         <v>421</v>
       </c>
-      <c r="H38" s="180"/>
-      <c r="I38" s="180"/>
-      <c r="J38" s="180"/>
-      <c r="K38" s="180"/>
-      <c r="L38" s="180"/>
-      <c r="M38" s="180"/>
-      <c r="N38" s="180"/>
-      <c r="O38" s="180"/>
-      <c r="P38" s="180"/>
-      <c r="Q38" s="180"/>
+      <c r="H38" s="191"/>
+      <c r="I38" s="191"/>
+      <c r="J38" s="191"/>
+      <c r="K38" s="191"/>
+      <c r="L38" s="191"/>
+      <c r="M38" s="191"/>
+      <c r="N38" s="191"/>
+      <c r="O38" s="191"/>
+      <c r="P38" s="191"/>
+      <c r="Q38" s="191"/>
       <c r="R38" s="109" t="s">
         <v>221</v>
       </c>
@@ -17643,20 +18021,20 @@
         <v>224</v>
       </c>
       <c r="E39" s="115"/>
-      <c r="F39" s="180" t="s">
+      <c r="F39" s="191" t="s">
         <v>424</v>
       </c>
-      <c r="G39" s="180"/>
-      <c r="H39" s="180"/>
-      <c r="I39" s="180"/>
-      <c r="J39" s="180"/>
-      <c r="K39" s="180"/>
-      <c r="L39" s="180"/>
-      <c r="M39" s="180"/>
-      <c r="N39" s="180"/>
-      <c r="O39" s="180"/>
-      <c r="P39" s="180"/>
-      <c r="Q39" s="180"/>
+      <c r="G39" s="191"/>
+      <c r="H39" s="191"/>
+      <c r="I39" s="191"/>
+      <c r="J39" s="191"/>
+      <c r="K39" s="191"/>
+      <c r="L39" s="191"/>
+      <c r="M39" s="191"/>
+      <c r="N39" s="191"/>
+      <c r="O39" s="191"/>
+      <c r="P39" s="191"/>
+      <c r="Q39" s="191"/>
       <c r="R39" s="109" t="s">
         <v>425</v>
       </c>
@@ -17678,21 +18056,21 @@
       <c r="F40" s="116" t="s">
         <v>430</v>
       </c>
-      <c r="G40" s="180" t="s">
+      <c r="G40" s="191" t="s">
         <v>431</v>
       </c>
-      <c r="H40" s="180"/>
+      <c r="H40" s="191"/>
       <c r="I40" s="117"/>
-      <c r="J40" s="180" t="s">
+      <c r="J40" s="191" t="s">
         <v>432</v>
       </c>
-      <c r="K40" s="180"/>
-      <c r="L40" s="180"/>
-      <c r="M40" s="180"/>
-      <c r="N40" s="180"/>
-      <c r="O40" s="180"/>
-      <c r="P40" s="180"/>
-      <c r="Q40" s="180"/>
+      <c r="K40" s="191"/>
+      <c r="L40" s="191"/>
+      <c r="M40" s="191"/>
+      <c r="N40" s="191"/>
+      <c r="O40" s="191"/>
+      <c r="P40" s="191"/>
+      <c r="Q40" s="191"/>
       <c r="S40" s="113" t="s">
         <v>433</v>
       </c>
@@ -17727,20 +18105,20 @@
         <v>436</v>
       </c>
       <c r="E42" s="115"/>
-      <c r="F42" s="195" t="s">
+      <c r="F42" s="206" t="s">
         <v>437</v>
       </c>
-      <c r="G42" s="180"/>
-      <c r="H42" s="180"/>
-      <c r="I42" s="180"/>
-      <c r="J42" s="180"/>
-      <c r="K42" s="180"/>
-      <c r="L42" s="180"/>
-      <c r="M42" s="180"/>
-      <c r="N42" s="180"/>
-      <c r="O42" s="180"/>
-      <c r="P42" s="180"/>
-      <c r="Q42" s="180"/>
+      <c r="G42" s="191"/>
+      <c r="H42" s="191"/>
+      <c r="I42" s="191"/>
+      <c r="J42" s="191"/>
+      <c r="K42" s="191"/>
+      <c r="L42" s="191"/>
+      <c r="M42" s="191"/>
+      <c r="N42" s="191"/>
+      <c r="O42" s="191"/>
+      <c r="P42" s="191"/>
+      <c r="Q42" s="191"/>
       <c r="R42" s="109" t="s">
         <v>221</v>
       </c>
@@ -17757,14 +18135,14 @@
         <v>224</v>
       </c>
       <c r="E43" s="115"/>
-      <c r="F43" s="180" t="s">
+      <c r="F43" s="191" t="s">
         <v>440</v>
       </c>
-      <c r="G43" s="180"/>
-      <c r="H43" s="180"/>
-      <c r="I43" s="180"/>
-      <c r="J43" s="180"/>
-      <c r="K43" s="180"/>
+      <c r="G43" s="191"/>
+      <c r="H43" s="191"/>
+      <c r="I43" s="191"/>
+      <c r="J43" s="191"/>
+      <c r="K43" s="191"/>
       <c r="L43" s="116" t="s">
         <v>441</v>
       </c>
@@ -17841,30 +18219,30 @@
         <v>458</v>
       </c>
       <c r="E45" s="115"/>
-      <c r="F45" s="180" t="s">
+      <c r="F45" s="191" t="s">
         <v>459</v>
       </c>
-      <c r="G45" s="180"/>
-      <c r="H45" s="180"/>
-      <c r="I45" s="180"/>
+      <c r="G45" s="191"/>
+      <c r="H45" s="191"/>
+      <c r="I45" s="191"/>
       <c r="J45" s="116" t="s">
         <v>460</v>
       </c>
       <c r="K45" s="116" t="s">
         <v>461</v>
       </c>
-      <c r="L45" s="180" t="s">
+      <c r="L45" s="191" t="s">
         <v>462</v>
       </c>
-      <c r="M45" s="180"/>
-      <c r="N45" s="195" t="s">
+      <c r="M45" s="191"/>
+      <c r="N45" s="206" t="s">
         <v>463</v>
       </c>
-      <c r="O45" s="195"/>
-      <c r="P45" s="180" t="s">
+      <c r="O45" s="206"/>
+      <c r="P45" s="191" t="s">
         <v>464</v>
       </c>
-      <c r="Q45" s="180"/>
+      <c r="Q45" s="191"/>
       <c r="R45" s="109" t="s">
         <v>221</v>
       </c>
@@ -17881,20 +18259,20 @@
         <v>224</v>
       </c>
       <c r="E46" s="115"/>
-      <c r="F46" s="180" t="s">
+      <c r="F46" s="191" t="s">
         <v>467</v>
       </c>
-      <c r="G46" s="180"/>
-      <c r="H46" s="180"/>
-      <c r="I46" s="180"/>
-      <c r="J46" s="180"/>
-      <c r="K46" s="180"/>
-      <c r="L46" s="180"/>
-      <c r="M46" s="180"/>
-      <c r="N46" s="180"/>
-      <c r="O46" s="180"/>
-      <c r="P46" s="180"/>
-      <c r="Q46" s="180"/>
+      <c r="G46" s="191"/>
+      <c r="H46" s="191"/>
+      <c r="I46" s="191"/>
+      <c r="J46" s="191"/>
+      <c r="K46" s="191"/>
+      <c r="L46" s="191"/>
+      <c r="M46" s="191"/>
+      <c r="N46" s="191"/>
+      <c r="O46" s="191"/>
+      <c r="P46" s="191"/>
+      <c r="Q46" s="191"/>
       <c r="R46" s="109" t="s">
         <v>221</v>
       </c>
@@ -17919,16 +18297,16 @@
       <c r="I47" s="117"/>
       <c r="J47" s="117"/>
       <c r="K47" s="117"/>
-      <c r="L47" s="179" t="s">
+      <c r="L47" s="190" t="s">
         <v>472</v>
       </c>
-      <c r="M47" s="179"/>
-      <c r="N47" s="180" t="s">
+      <c r="M47" s="190"/>
+      <c r="N47" s="191" t="s">
         <v>473</v>
       </c>
-      <c r="O47" s="180"/>
-      <c r="P47" s="180"/>
-      <c r="Q47" s="180"/>
+      <c r="O47" s="191"/>
+      <c r="P47" s="191"/>
+      <c r="Q47" s="191"/>
       <c r="R47" s="109" t="s">
         <v>474</v>
       </c>
@@ -17954,17 +18332,17 @@
       <c r="H48" s="123"/>
       <c r="I48" s="123"/>
       <c r="J48" s="123"/>
-      <c r="K48" s="179" t="s">
+      <c r="K48" s="190" t="s">
         <v>479</v>
       </c>
-      <c r="L48" s="179"/>
-      <c r="M48" s="179"/>
+      <c r="L48" s="190"/>
+      <c r="M48" s="190"/>
       <c r="N48" s="123"/>
-      <c r="O48" s="179" t="s">
+      <c r="O48" s="190" t="s">
         <v>480</v>
       </c>
-      <c r="P48" s="179"/>
-      <c r="Q48" s="179"/>
+      <c r="P48" s="190"/>
+      <c r="Q48" s="190"/>
       <c r="R48" s="109" t="s">
         <v>221</v>
       </c>
@@ -18079,16 +18457,16 @@
       <c r="F53" s="116" t="s">
         <v>491</v>
       </c>
-      <c r="G53" s="179" t="s">
+      <c r="G53" s="190" t="s">
         <v>492</v>
       </c>
-      <c r="H53" s="179"/>
-      <c r="I53" s="179"/>
-      <c r="J53" s="194" t="s">
+      <c r="H53" s="190"/>
+      <c r="I53" s="190"/>
+      <c r="J53" s="205" t="s">
         <v>493</v>
       </c>
-      <c r="K53" s="185"/>
-      <c r="L53" s="184"/>
+      <c r="K53" s="196"/>
+      <c r="L53" s="195"/>
       <c r="M53" s="116" t="s">
         <v>494</v>
       </c>
@@ -18130,12 +18508,12 @@
       <c r="K54" s="117"/>
       <c r="L54" s="117"/>
       <c r="M54" s="117"/>
-      <c r="N54" s="180" t="s">
+      <c r="N54" s="191" t="s">
         <v>503</v>
       </c>
-      <c r="O54" s="180"/>
-      <c r="P54" s="180"/>
-      <c r="Q54" s="180"/>
+      <c r="O54" s="191"/>
+      <c r="P54" s="191"/>
+      <c r="Q54" s="191"/>
       <c r="R54" s="109" t="s">
         <v>221</v>
       </c>
@@ -18152,20 +18530,20 @@
         <v>506</v>
       </c>
       <c r="E55" s="115"/>
-      <c r="F55" s="180" t="s">
+      <c r="F55" s="191" t="s">
         <v>507</v>
       </c>
-      <c r="G55" s="180"/>
-      <c r="H55" s="180"/>
-      <c r="I55" s="180"/>
-      <c r="J55" s="180"/>
-      <c r="K55" s="180"/>
-      <c r="L55" s="180"/>
-      <c r="M55" s="180"/>
-      <c r="N55" s="180"/>
-      <c r="O55" s="180"/>
-      <c r="P55" s="180"/>
-      <c r="Q55" s="180"/>
+      <c r="G55" s="191"/>
+      <c r="H55" s="191"/>
+      <c r="I55" s="191"/>
+      <c r="J55" s="191"/>
+      <c r="K55" s="191"/>
+      <c r="L55" s="191"/>
+      <c r="M55" s="191"/>
+      <c r="N55" s="191"/>
+      <c r="O55" s="191"/>
+      <c r="P55" s="191"/>
+      <c r="Q55" s="191"/>
       <c r="R55" s="109" t="s">
         <v>221</v>
       </c>
@@ -18188,16 +18566,16 @@
       <c r="I56" s="117"/>
       <c r="J56" s="117"/>
       <c r="K56" s="117"/>
-      <c r="L56" s="180" t="s">
+      <c r="L56" s="191" t="s">
         <v>511</v>
       </c>
-      <c r="M56" s="180"/>
-      <c r="N56" s="180" t="s">
+      <c r="M56" s="191"/>
+      <c r="N56" s="191" t="s">
         <v>512</v>
       </c>
-      <c r="O56" s="180"/>
-      <c r="P56" s="180"/>
-      <c r="Q56" s="180"/>
+      <c r="O56" s="191"/>
+      <c r="P56" s="191"/>
+      <c r="Q56" s="191"/>
       <c r="R56" s="109" t="s">
         <v>221</v>
       </c>
@@ -18248,20 +18626,20 @@
         <v>520</v>
       </c>
       <c r="E58" s="115"/>
-      <c r="F58" s="180" t="s">
+      <c r="F58" s="191" t="s">
         <v>521</v>
       </c>
-      <c r="G58" s="180"/>
-      <c r="H58" s="180"/>
-      <c r="I58" s="180"/>
-      <c r="J58" s="180"/>
-      <c r="K58" s="180"/>
-      <c r="L58" s="180"/>
-      <c r="M58" s="180"/>
-      <c r="N58" s="180"/>
-      <c r="O58" s="180"/>
-      <c r="P58" s="180"/>
-      <c r="Q58" s="180"/>
+      <c r="G58" s="191"/>
+      <c r="H58" s="191"/>
+      <c r="I58" s="191"/>
+      <c r="J58" s="191"/>
+      <c r="K58" s="191"/>
+      <c r="L58" s="191"/>
+      <c r="M58" s="191"/>
+      <c r="N58" s="191"/>
+      <c r="O58" s="191"/>
+      <c r="P58" s="191"/>
+      <c r="Q58" s="191"/>
       <c r="R58" s="109" t="s">
         <v>221</v>
       </c>
@@ -18358,16 +18736,16 @@
       <c r="G63" s="123"/>
       <c r="H63" s="123"/>
       <c r="I63" s="123"/>
-      <c r="J63" s="196" t="s">
+      <c r="J63" s="207" t="s">
         <v>523</v>
       </c>
-      <c r="K63" s="196"/>
-      <c r="L63" s="196"/>
-      <c r="M63" s="196"/>
-      <c r="N63" s="196"/>
-      <c r="O63" s="196"/>
-      <c r="P63" s="196"/>
-      <c r="Q63" s="196"/>
+      <c r="K63" s="207"/>
+      <c r="L63" s="207"/>
+      <c r="M63" s="207"/>
+      <c r="N63" s="207"/>
+      <c r="O63" s="207"/>
+      <c r="P63" s="207"/>
+      <c r="Q63" s="207"/>
       <c r="S63" s="113"/>
     </row>
     <row r="64" spans="2:19" x14ac:dyDescent="0.45">
@@ -18381,20 +18759,20 @@
       <c r="E64" s="115"/>
       <c r="F64" s="135"/>
       <c r="G64" s="135"/>
-      <c r="H64" s="196" t="s">
+      <c r="H64" s="207" t="s">
         <v>525</v>
       </c>
-      <c r="I64" s="197"/>
-      <c r="J64" s="197"/>
-      <c r="K64" s="197"/>
-      <c r="L64" s="197"/>
-      <c r="M64" s="196" t="s">
+      <c r="I64" s="208"/>
+      <c r="J64" s="208"/>
+      <c r="K64" s="208"/>
+      <c r="L64" s="208"/>
+      <c r="M64" s="207" t="s">
         <v>526</v>
       </c>
-      <c r="N64" s="197"/>
-      <c r="O64" s="197"/>
-      <c r="P64" s="197"/>
-      <c r="Q64" s="197"/>
+      <c r="N64" s="208"/>
+      <c r="O64" s="208"/>
+      <c r="P64" s="208"/>
+      <c r="Q64" s="208"/>
       <c r="S64" s="113"/>
     </row>
     <row r="65" spans="2:19" x14ac:dyDescent="0.45">
@@ -18406,22 +18784,22 @@
         <v>527</v>
       </c>
       <c r="E65" s="115"/>
-      <c r="F65" s="198" t="s">
+      <c r="F65" s="209" t="s">
         <v>528</v>
       </c>
-      <c r="G65" s="199"/>
-      <c r="H65" s="199"/>
-      <c r="I65" s="199"/>
-      <c r="J65" s="200"/>
+      <c r="G65" s="210"/>
+      <c r="H65" s="210"/>
+      <c r="I65" s="210"/>
+      <c r="J65" s="211"/>
       <c r="K65" s="123"/>
       <c r="L65" s="123"/>
-      <c r="M65" s="198" t="s">
+      <c r="M65" s="209" t="s">
         <v>529</v>
       </c>
-      <c r="N65" s="199"/>
-      <c r="O65" s="199"/>
-      <c r="P65" s="199"/>
-      <c r="Q65" s="200"/>
+      <c r="N65" s="210"/>
+      <c r="O65" s="210"/>
+      <c r="P65" s="210"/>
+      <c r="Q65" s="211"/>
       <c r="S65" s="113"/>
     </row>
     <row r="66" spans="2:19" x14ac:dyDescent="0.45">
@@ -18437,18 +18815,18 @@
       <c r="G66" s="123"/>
       <c r="H66" s="123"/>
       <c r="I66" s="123"/>
-      <c r="J66" s="196" t="s">
+      <c r="J66" s="207" t="s">
         <v>530</v>
       </c>
-      <c r="K66" s="196"/>
-      <c r="L66" s="196"/>
-      <c r="M66" s="196"/>
-      <c r="N66" s="196" t="s">
+      <c r="K66" s="207"/>
+      <c r="L66" s="207"/>
+      <c r="M66" s="207"/>
+      <c r="N66" s="207" t="s">
         <v>531</v>
       </c>
-      <c r="O66" s="196"/>
-      <c r="P66" s="196"/>
-      <c r="Q66" s="196"/>
+      <c r="O66" s="207"/>
+      <c r="P66" s="207"/>
+      <c r="Q66" s="207"/>
       <c r="S66" s="113"/>
     </row>
     <row r="67" spans="2:19" x14ac:dyDescent="0.45">
@@ -18463,17 +18841,17 @@
       <c r="F67" s="123"/>
       <c r="G67" s="123"/>
       <c r="H67" s="123"/>
-      <c r="I67" s="198" t="s">
+      <c r="I67" s="209" t="s">
         <v>532</v>
       </c>
-      <c r="J67" s="199"/>
-      <c r="K67" s="199"/>
-      <c r="L67" s="199"/>
-      <c r="M67" s="199"/>
-      <c r="N67" s="199"/>
-      <c r="O67" s="199"/>
-      <c r="P67" s="199"/>
-      <c r="Q67" s="200"/>
+      <c r="J67" s="210"/>
+      <c r="K67" s="210"/>
+      <c r="L67" s="210"/>
+      <c r="M67" s="210"/>
+      <c r="N67" s="210"/>
+      <c r="O67" s="210"/>
+      <c r="P67" s="210"/>
+      <c r="Q67" s="211"/>
       <c r="S67" s="113"/>
     </row>
     <row r="68" spans="2:19" x14ac:dyDescent="0.45">
@@ -18488,17 +18866,17 @@
       <c r="F68" s="123"/>
       <c r="G68" s="123"/>
       <c r="H68" s="123"/>
-      <c r="I68" s="198" t="s">
+      <c r="I68" s="209" t="s">
         <v>533</v>
       </c>
-      <c r="J68" s="199"/>
-      <c r="K68" s="199"/>
-      <c r="L68" s="199"/>
-      <c r="M68" s="199"/>
-      <c r="N68" s="199"/>
-      <c r="O68" s="199"/>
-      <c r="P68" s="199"/>
-      <c r="Q68" s="200"/>
+      <c r="J68" s="210"/>
+      <c r="K68" s="210"/>
+      <c r="L68" s="210"/>
+      <c r="M68" s="210"/>
+      <c r="N68" s="210"/>
+      <c r="O68" s="210"/>
+      <c r="P68" s="210"/>
+      <c r="Q68" s="211"/>
       <c r="S68" s="113"/>
     </row>
     <row r="69" spans="2:19" x14ac:dyDescent="0.45">
@@ -18513,17 +18891,17 @@
       <c r="F69" s="123"/>
       <c r="G69" s="123"/>
       <c r="H69" s="123"/>
-      <c r="I69" s="198" t="s">
+      <c r="I69" s="209" t="s">
         <v>534</v>
       </c>
-      <c r="J69" s="199"/>
-      <c r="K69" s="199"/>
-      <c r="L69" s="199"/>
-      <c r="M69" s="199"/>
-      <c r="N69" s="199"/>
-      <c r="O69" s="199"/>
-      <c r="P69" s="199"/>
-      <c r="Q69" s="200"/>
+      <c r="J69" s="210"/>
+      <c r="K69" s="210"/>
+      <c r="L69" s="210"/>
+      <c r="M69" s="210"/>
+      <c r="N69" s="210"/>
+      <c r="O69" s="210"/>
+      <c r="P69" s="210"/>
+      <c r="Q69" s="211"/>
       <c r="S69" s="113"/>
     </row>
     <row r="70" spans="2:19" x14ac:dyDescent="0.45">
@@ -18538,17 +18916,17 @@
       <c r="F70" s="123"/>
       <c r="G70" s="123"/>
       <c r="H70" s="123"/>
-      <c r="I70" s="198" t="s">
+      <c r="I70" s="209" t="s">
         <v>536</v>
       </c>
-      <c r="J70" s="199"/>
-      <c r="K70" s="199"/>
-      <c r="L70" s="199"/>
-      <c r="M70" s="199"/>
-      <c r="N70" s="199"/>
-      <c r="O70" s="199"/>
-      <c r="P70" s="199"/>
-      <c r="Q70" s="200"/>
+      <c r="J70" s="210"/>
+      <c r="K70" s="210"/>
+      <c r="L70" s="210"/>
+      <c r="M70" s="210"/>
+      <c r="N70" s="210"/>
+      <c r="O70" s="210"/>
+      <c r="P70" s="210"/>
+      <c r="Q70" s="211"/>
       <c r="S70" s="113"/>
     </row>
     <row r="71" spans="2:19" x14ac:dyDescent="0.45">
@@ -18563,17 +18941,17 @@
       <c r="F71" s="123"/>
       <c r="G71" s="123"/>
       <c r="H71" s="123"/>
-      <c r="I71" s="198" t="s">
+      <c r="I71" s="209" t="s">
         <v>538</v>
       </c>
-      <c r="J71" s="199"/>
-      <c r="K71" s="199"/>
-      <c r="L71" s="199"/>
-      <c r="M71" s="199"/>
-      <c r="N71" s="199"/>
-      <c r="O71" s="199"/>
-      <c r="P71" s="199"/>
-      <c r="Q71" s="200"/>
+      <c r="J71" s="210"/>
+      <c r="K71" s="210"/>
+      <c r="L71" s="210"/>
+      <c r="M71" s="210"/>
+      <c r="N71" s="210"/>
+      <c r="O71" s="210"/>
+      <c r="P71" s="210"/>
+      <c r="Q71" s="211"/>
       <c r="S71" s="113"/>
     </row>
     <row r="72" spans="2:19" x14ac:dyDescent="0.45">
@@ -18588,17 +18966,17 @@
       <c r="F72" s="123"/>
       <c r="G72" s="123"/>
       <c r="H72" s="123"/>
-      <c r="I72" s="198" t="s">
+      <c r="I72" s="209" t="s">
         <v>539</v>
       </c>
-      <c r="J72" s="199"/>
-      <c r="K72" s="199"/>
-      <c r="L72" s="199"/>
-      <c r="M72" s="199"/>
-      <c r="N72" s="199"/>
-      <c r="O72" s="199"/>
-      <c r="P72" s="199"/>
-      <c r="Q72" s="200"/>
+      <c r="J72" s="210"/>
+      <c r="K72" s="210"/>
+      <c r="L72" s="210"/>
+      <c r="M72" s="210"/>
+      <c r="N72" s="210"/>
+      <c r="O72" s="210"/>
+      <c r="P72" s="210"/>
+      <c r="Q72" s="211"/>
       <c r="S72" s="113"/>
     </row>
     <row r="73" spans="2:19" x14ac:dyDescent="0.45">
@@ -18613,17 +18991,17 @@
       <c r="F73" s="123"/>
       <c r="G73" s="123"/>
       <c r="H73" s="123"/>
-      <c r="I73" s="198" t="s">
+      <c r="I73" s="209" t="s">
         <v>540</v>
       </c>
-      <c r="J73" s="199"/>
-      <c r="K73" s="199"/>
-      <c r="L73" s="199"/>
-      <c r="M73" s="199"/>
-      <c r="N73" s="199"/>
-      <c r="O73" s="199"/>
-      <c r="P73" s="199"/>
-      <c r="Q73" s="200"/>
+      <c r="J73" s="210"/>
+      <c r="K73" s="210"/>
+      <c r="L73" s="210"/>
+      <c r="M73" s="210"/>
+      <c r="N73" s="210"/>
+      <c r="O73" s="210"/>
+      <c r="P73" s="210"/>
+      <c r="Q73" s="211"/>
       <c r="S73" s="113"/>
     </row>
     <row r="74" spans="2:19" x14ac:dyDescent="0.45">
@@ -18638,17 +19016,17 @@
       <c r="F74" s="123"/>
       <c r="G74" s="123"/>
       <c r="H74" s="123"/>
-      <c r="I74" s="198" t="s">
+      <c r="I74" s="209" t="s">
         <v>541</v>
       </c>
-      <c r="J74" s="199"/>
-      <c r="K74" s="199"/>
-      <c r="L74" s="199"/>
-      <c r="M74" s="199"/>
-      <c r="N74" s="199"/>
-      <c r="O74" s="199"/>
-      <c r="P74" s="199"/>
-      <c r="Q74" s="200"/>
+      <c r="J74" s="210"/>
+      <c r="K74" s="210"/>
+      <c r="L74" s="210"/>
+      <c r="M74" s="210"/>
+      <c r="N74" s="210"/>
+      <c r="O74" s="210"/>
+      <c r="P74" s="210"/>
+      <c r="Q74" s="211"/>
       <c r="S74" s="113"/>
     </row>
     <row r="75" spans="2:19" x14ac:dyDescent="0.45">
@@ -18663,17 +19041,17 @@
       <c r="F75" s="123"/>
       <c r="G75" s="123"/>
       <c r="H75" s="123"/>
-      <c r="I75" s="198" t="s">
+      <c r="I75" s="209" t="s">
         <v>542</v>
       </c>
-      <c r="J75" s="199"/>
-      <c r="K75" s="199"/>
-      <c r="L75" s="199"/>
-      <c r="M75" s="199"/>
-      <c r="N75" s="199"/>
-      <c r="O75" s="199"/>
-      <c r="P75" s="199"/>
-      <c r="Q75" s="200"/>
+      <c r="J75" s="210"/>
+      <c r="K75" s="210"/>
+      <c r="L75" s="210"/>
+      <c r="M75" s="210"/>
+      <c r="N75" s="210"/>
+      <c r="O75" s="210"/>
+      <c r="P75" s="210"/>
+      <c r="Q75" s="211"/>
       <c r="S75" s="113"/>
     </row>
     <row r="76" spans="2:19" x14ac:dyDescent="0.45">
@@ -18688,17 +19066,17 @@
       <c r="F76" s="123"/>
       <c r="G76" s="123"/>
       <c r="H76" s="123"/>
-      <c r="I76" s="198" t="s">
+      <c r="I76" s="209" t="s">
         <v>543</v>
       </c>
-      <c r="J76" s="199"/>
-      <c r="K76" s="199"/>
-      <c r="L76" s="199"/>
-      <c r="M76" s="199"/>
-      <c r="N76" s="199"/>
-      <c r="O76" s="199"/>
-      <c r="P76" s="199"/>
-      <c r="Q76" s="200"/>
+      <c r="J76" s="210"/>
+      <c r="K76" s="210"/>
+      <c r="L76" s="210"/>
+      <c r="M76" s="210"/>
+      <c r="N76" s="210"/>
+      <c r="O76" s="210"/>
+      <c r="P76" s="210"/>
+      <c r="Q76" s="211"/>
       <c r="S76" s="113"/>
     </row>
     <row r="77" spans="2:19" x14ac:dyDescent="0.45">
@@ -18713,17 +19091,17 @@
       <c r="F77" s="123"/>
       <c r="G77" s="123"/>
       <c r="H77" s="123"/>
-      <c r="I77" s="198" t="s">
+      <c r="I77" s="209" t="s">
         <v>544</v>
       </c>
-      <c r="J77" s="199"/>
-      <c r="K77" s="199"/>
-      <c r="L77" s="199"/>
-      <c r="M77" s="199"/>
-      <c r="N77" s="199"/>
-      <c r="O77" s="199"/>
-      <c r="P77" s="199"/>
-      <c r="Q77" s="200"/>
+      <c r="J77" s="210"/>
+      <c r="K77" s="210"/>
+      <c r="L77" s="210"/>
+      <c r="M77" s="210"/>
+      <c r="N77" s="210"/>
+      <c r="O77" s="210"/>
+      <c r="P77" s="210"/>
+      <c r="Q77" s="211"/>
       <c r="S77" s="113"/>
     </row>
     <row r="78" spans="2:19" x14ac:dyDescent="0.45">
@@ -18738,17 +19116,17 @@
       <c r="F78" s="123"/>
       <c r="G78" s="123"/>
       <c r="H78" s="123"/>
-      <c r="I78" s="198" t="s">
+      <c r="I78" s="209" t="s">
         <v>545</v>
       </c>
-      <c r="J78" s="199"/>
-      <c r="K78" s="199"/>
-      <c r="L78" s="199"/>
-      <c r="M78" s="199"/>
-      <c r="N78" s="199"/>
-      <c r="O78" s="199"/>
-      <c r="P78" s="199"/>
-      <c r="Q78" s="200"/>
+      <c r="J78" s="210"/>
+      <c r="K78" s="210"/>
+      <c r="L78" s="210"/>
+      <c r="M78" s="210"/>
+      <c r="N78" s="210"/>
+      <c r="O78" s="210"/>
+      <c r="P78" s="210"/>
+      <c r="Q78" s="211"/>
       <c r="S78" s="113"/>
     </row>
     <row r="79" spans="2:19" x14ac:dyDescent="0.45">
@@ -18765,15 +19143,15 @@
       <c r="H79" s="123"/>
       <c r="I79" s="123"/>
       <c r="J79" s="123"/>
-      <c r="K79" s="198" t="s">
+      <c r="K79" s="209" t="s">
         <v>547</v>
       </c>
-      <c r="L79" s="199"/>
-      <c r="M79" s="199"/>
-      <c r="N79" s="199"/>
-      <c r="O79" s="199"/>
-      <c r="P79" s="199"/>
-      <c r="Q79" s="200"/>
+      <c r="L79" s="210"/>
+      <c r="M79" s="210"/>
+      <c r="N79" s="210"/>
+      <c r="O79" s="210"/>
+      <c r="P79" s="210"/>
+      <c r="Q79" s="211"/>
       <c r="S79" s="113"/>
     </row>
     <row r="80" spans="2:19" x14ac:dyDescent="0.45">
@@ -18790,15 +19168,15 @@
       <c r="H80" s="123"/>
       <c r="I80" s="123"/>
       <c r="J80" s="123"/>
-      <c r="K80" s="198" t="s">
+      <c r="K80" s="209" t="s">
         <v>548</v>
       </c>
-      <c r="L80" s="199"/>
-      <c r="M80" s="199"/>
-      <c r="N80" s="199"/>
-      <c r="O80" s="199"/>
-      <c r="P80" s="199"/>
-      <c r="Q80" s="200"/>
+      <c r="L80" s="210"/>
+      <c r="M80" s="210"/>
+      <c r="N80" s="210"/>
+      <c r="O80" s="210"/>
+      <c r="P80" s="210"/>
+      <c r="Q80" s="211"/>
       <c r="S80" s="113"/>
     </row>
     <row r="81" spans="2:19" x14ac:dyDescent="0.45">
@@ -18815,15 +19193,15 @@
       <c r="H81" s="123"/>
       <c r="I81" s="123"/>
       <c r="J81" s="123"/>
-      <c r="K81" s="198" t="s">
+      <c r="K81" s="209" t="s">
         <v>550</v>
       </c>
-      <c r="L81" s="199"/>
-      <c r="M81" s="199"/>
-      <c r="N81" s="199"/>
-      <c r="O81" s="199"/>
-      <c r="P81" s="199"/>
-      <c r="Q81" s="200"/>
+      <c r="L81" s="210"/>
+      <c r="M81" s="210"/>
+      <c r="N81" s="210"/>
+      <c r="O81" s="210"/>
+      <c r="P81" s="210"/>
+      <c r="Q81" s="211"/>
       <c r="S81" s="113"/>
     </row>
     <row r="82" spans="2:19" x14ac:dyDescent="0.45">
@@ -18840,15 +19218,15 @@
       <c r="H82" s="123"/>
       <c r="I82" s="123"/>
       <c r="J82" s="123"/>
-      <c r="K82" s="198" t="s">
+      <c r="K82" s="209" t="s">
         <v>551</v>
       </c>
-      <c r="L82" s="199"/>
-      <c r="M82" s="199"/>
-      <c r="N82" s="199"/>
-      <c r="O82" s="199"/>
-      <c r="P82" s="199"/>
-      <c r="Q82" s="200"/>
+      <c r="L82" s="210"/>
+      <c r="M82" s="210"/>
+      <c r="N82" s="210"/>
+      <c r="O82" s="210"/>
+      <c r="P82" s="210"/>
+      <c r="Q82" s="211"/>
       <c r="S82" s="113"/>
     </row>
     <row r="83" spans="2:19" x14ac:dyDescent="0.45">
@@ -18865,15 +19243,15 @@
       <c r="H83" s="123"/>
       <c r="I83" s="123"/>
       <c r="J83" s="123"/>
-      <c r="K83" s="198" t="s">
+      <c r="K83" s="209" t="s">
         <v>552</v>
       </c>
-      <c r="L83" s="199"/>
-      <c r="M83" s="199"/>
-      <c r="N83" s="199"/>
-      <c r="O83" s="199"/>
-      <c r="P83" s="199"/>
-      <c r="Q83" s="200"/>
+      <c r="L83" s="210"/>
+      <c r="M83" s="210"/>
+      <c r="N83" s="210"/>
+      <c r="O83" s="210"/>
+      <c r="P83" s="210"/>
+      <c r="Q83" s="211"/>
       <c r="S83" s="113"/>
     </row>
     <row r="84" spans="2:19" x14ac:dyDescent="0.45">
@@ -18890,15 +19268,15 @@
       <c r="H84" s="123"/>
       <c r="I84" s="123"/>
       <c r="J84" s="123"/>
-      <c r="K84" s="198" t="s">
+      <c r="K84" s="209" t="s">
         <v>553</v>
       </c>
-      <c r="L84" s="199"/>
-      <c r="M84" s="199"/>
-      <c r="N84" s="199"/>
-      <c r="O84" s="199"/>
-      <c r="P84" s="199"/>
-      <c r="Q84" s="200"/>
+      <c r="L84" s="210"/>
+      <c r="M84" s="210"/>
+      <c r="N84" s="210"/>
+      <c r="O84" s="210"/>
+      <c r="P84" s="210"/>
+      <c r="Q84" s="211"/>
       <c r="S84" s="113"/>
     </row>
     <row r="85" spans="2:19" x14ac:dyDescent="0.45">
@@ -18915,15 +19293,15 @@
       <c r="H85" s="123"/>
       <c r="I85" s="123"/>
       <c r="J85" s="123"/>
-      <c r="K85" s="198" t="s">
+      <c r="K85" s="209" t="s">
         <v>555</v>
       </c>
-      <c r="L85" s="199"/>
-      <c r="M85" s="199"/>
-      <c r="N85" s="199"/>
-      <c r="O85" s="199"/>
-      <c r="P85" s="199"/>
-      <c r="Q85" s="200"/>
+      <c r="L85" s="210"/>
+      <c r="M85" s="210"/>
+      <c r="N85" s="210"/>
+      <c r="O85" s="210"/>
+      <c r="P85" s="210"/>
+      <c r="Q85" s="211"/>
       <c r="S85" s="113"/>
     </row>
     <row r="86" spans="2:19" x14ac:dyDescent="0.45">
@@ -18940,15 +19318,15 @@
       <c r="H86" s="123"/>
       <c r="I86" s="123"/>
       <c r="J86" s="123"/>
-      <c r="K86" s="198" t="s">
+      <c r="K86" s="209" t="s">
         <v>557</v>
       </c>
-      <c r="L86" s="199"/>
-      <c r="M86" s="199"/>
-      <c r="N86" s="199"/>
-      <c r="O86" s="199"/>
-      <c r="P86" s="199"/>
-      <c r="Q86" s="200"/>
+      <c r="L86" s="210"/>
+      <c r="M86" s="210"/>
+      <c r="N86" s="210"/>
+      <c r="O86" s="210"/>
+      <c r="P86" s="210"/>
+      <c r="Q86" s="211"/>
       <c r="S86" s="113"/>
     </row>
     <row r="87" spans="2:19" x14ac:dyDescent="0.45">
@@ -18965,15 +19343,15 @@
       <c r="H87" s="123"/>
       <c r="I87" s="123"/>
       <c r="J87" s="123"/>
-      <c r="K87" s="198" t="s">
+      <c r="K87" s="209" t="s">
         <v>559</v>
       </c>
-      <c r="L87" s="199"/>
-      <c r="M87" s="199"/>
-      <c r="N87" s="199"/>
-      <c r="O87" s="199"/>
-      <c r="P87" s="199"/>
-      <c r="Q87" s="200"/>
+      <c r="L87" s="210"/>
+      <c r="M87" s="210"/>
+      <c r="N87" s="210"/>
+      <c r="O87" s="210"/>
+      <c r="P87" s="210"/>
+      <c r="Q87" s="211"/>
       <c r="S87" s="113"/>
     </row>
     <row r="88" spans="2:19" x14ac:dyDescent="0.45">
@@ -18990,15 +19368,15 @@
       <c r="H88" s="123"/>
       <c r="I88" s="123"/>
       <c r="J88" s="123"/>
-      <c r="K88" s="198" t="s">
+      <c r="K88" s="209" t="s">
         <v>561</v>
       </c>
-      <c r="L88" s="199"/>
-      <c r="M88" s="199"/>
-      <c r="N88" s="199"/>
-      <c r="O88" s="199"/>
-      <c r="P88" s="199"/>
-      <c r="Q88" s="200"/>
+      <c r="L88" s="210"/>
+      <c r="M88" s="210"/>
+      <c r="N88" s="210"/>
+      <c r="O88" s="210"/>
+      <c r="P88" s="210"/>
+      <c r="Q88" s="211"/>
       <c r="S88" s="113"/>
     </row>
     <row r="89" spans="2:19" x14ac:dyDescent="0.45">
@@ -19015,15 +19393,15 @@
       <c r="H89" s="123"/>
       <c r="I89" s="123"/>
       <c r="J89" s="123"/>
-      <c r="K89" s="198" t="s">
+      <c r="K89" s="209" t="s">
         <v>562</v>
       </c>
-      <c r="L89" s="199"/>
-      <c r="M89" s="199"/>
-      <c r="N89" s="199"/>
-      <c r="O89" s="199"/>
-      <c r="P89" s="199"/>
-      <c r="Q89" s="200"/>
+      <c r="L89" s="210"/>
+      <c r="M89" s="210"/>
+      <c r="N89" s="210"/>
+      <c r="O89" s="210"/>
+      <c r="P89" s="210"/>
+      <c r="Q89" s="211"/>
       <c r="S89" s="113"/>
     </row>
     <row r="90" spans="2:19" x14ac:dyDescent="0.45">
@@ -19040,15 +19418,15 @@
       <c r="H90" s="123"/>
       <c r="I90" s="123"/>
       <c r="J90" s="123"/>
-      <c r="K90" s="198" t="s">
+      <c r="K90" s="209" t="s">
         <v>563</v>
       </c>
-      <c r="L90" s="199"/>
-      <c r="M90" s="199"/>
-      <c r="N90" s="199"/>
-      <c r="O90" s="199"/>
-      <c r="P90" s="199"/>
-      <c r="Q90" s="200"/>
+      <c r="L90" s="210"/>
+      <c r="M90" s="210"/>
+      <c r="N90" s="210"/>
+      <c r="O90" s="210"/>
+      <c r="P90" s="210"/>
+      <c r="Q90" s="211"/>
       <c r="S90" s="113"/>
     </row>
     <row r="91" spans="2:19" x14ac:dyDescent="0.45">
@@ -19060,20 +19438,20 @@
         <v>224</v>
       </c>
       <c r="E91" s="115"/>
-      <c r="F91" s="196" t="s">
+      <c r="F91" s="207" t="s">
         <v>564</v>
       </c>
-      <c r="G91" s="196"/>
-      <c r="H91" s="196"/>
-      <c r="I91" s="196"/>
-      <c r="J91" s="196"/>
-      <c r="K91" s="196"/>
-      <c r="L91" s="196"/>
-      <c r="M91" s="196"/>
-      <c r="N91" s="196"/>
-      <c r="O91" s="196"/>
-      <c r="P91" s="196"/>
-      <c r="Q91" s="196"/>
+      <c r="G91" s="207"/>
+      <c r="H91" s="207"/>
+      <c r="I91" s="207"/>
+      <c r="J91" s="207"/>
+      <c r="K91" s="207"/>
+      <c r="L91" s="207"/>
+      <c r="M91" s="207"/>
+      <c r="N91" s="207"/>
+      <c r="O91" s="207"/>
+      <c r="P91" s="207"/>
+      <c r="Q91" s="207"/>
       <c r="S91" s="113"/>
     </row>
     <row r="92" spans="2:19" x14ac:dyDescent="0.45">
@@ -19085,20 +19463,20 @@
         <v>224</v>
       </c>
       <c r="E92" s="115"/>
-      <c r="F92" s="196" t="s">
+      <c r="F92" s="207" t="s">
         <v>565</v>
       </c>
-      <c r="G92" s="196"/>
-      <c r="H92" s="196"/>
-      <c r="I92" s="196"/>
-      <c r="J92" s="196"/>
-      <c r="K92" s="196"/>
-      <c r="L92" s="196"/>
-      <c r="M92" s="196"/>
-      <c r="N92" s="196"/>
-      <c r="O92" s="196"/>
-      <c r="P92" s="196"/>
-      <c r="Q92" s="196"/>
+      <c r="G92" s="207"/>
+      <c r="H92" s="207"/>
+      <c r="I92" s="207"/>
+      <c r="J92" s="207"/>
+      <c r="K92" s="207"/>
+      <c r="L92" s="207"/>
+      <c r="M92" s="207"/>
+      <c r="N92" s="207"/>
+      <c r="O92" s="207"/>
+      <c r="P92" s="207"/>
+      <c r="Q92" s="207"/>
       <c r="S92" s="113"/>
     </row>
   </sheetData>
@@ -19224,7 +19602,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8955C504-3FEB-499A-A6D9-660B7C48D170}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
@@ -19263,7 +19641,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0408BB74-E718-448A-B466-1CBF5516D7A7}">
   <dimension ref="C24:D27"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
@@ -19275,34 +19653,34 @@
   <sheetData>
     <row r="24" spans="3:4" x14ac:dyDescent="0.45">
       <c r="C24" s="136" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="D24" s="136" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
     </row>
     <row r="25" spans="3:4" x14ac:dyDescent="0.45">
       <c r="C25" s="136" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="D25" s="136" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
     </row>
     <row r="26" spans="3:4" x14ac:dyDescent="0.45">
       <c r="C26" s="136" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="D26" s="136" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
     </row>
     <row r="27" spans="3:4" x14ac:dyDescent="0.45">
       <c r="C27" s="136" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="D27" s="136" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
     </row>
   </sheetData>
@@ -19340,7 +19718,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{176E8790-74D9-4A6F-962A-C28A733F4069}">
   <dimension ref="C3:E16"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
@@ -19351,46 +19729,46 @@
   <sheetData>
     <row r="3" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C3" s="137" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="D3" s="113">
         <v>20</v>
       </c>
       <c r="E3" s="113" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
     </row>
     <row r="4" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C4" s="137" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="D4" s="113">
         <v>16</v>
       </c>
       <c r="E4" s="113" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
     </row>
     <row r="5" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C5" s="137" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="D5" s="113">
         <v>5.0000000000000001E-3</v>
       </c>
       <c r="E5" s="113" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
     </row>
     <row r="6" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C6" s="137" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="D6" s="113">
         <v>8.3332999999999995</v>
       </c>
       <c r="E6" s="113" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
     </row>
     <row r="7" spans="3:5" x14ac:dyDescent="0.45">
@@ -19400,79 +19778,79 @@
     </row>
     <row r="8" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C8" s="137" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="D8" s="113">
         <f>D6-D4*D5*2</f>
         <v>8.1732999999999993</v>
       </c>
       <c r="E8" s="113" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
     </row>
     <row r="9" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C9" s="137" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="D9" s="113">
         <f>D6-D4*D5</f>
         <v>8.2532999999999994</v>
       </c>
       <c r="E9" s="113" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
     </row>
     <row r="10" spans="3:5" ht="34" x14ac:dyDescent="0.45">
       <c r="C10" s="138" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="D10" s="113">
         <f>D8/(D4*2)</f>
         <v>0.25541562499999998</v>
       </c>
       <c r="E10" s="113" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
     </row>
     <row r="11" spans="3:5" ht="34" x14ac:dyDescent="0.45">
       <c r="C11" s="138" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="D11" s="113">
         <f>D9/(D4)</f>
         <v>0.51583124999999996</v>
       </c>
       <c r="E11" s="113" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
     </row>
     <row r="12" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C12" s="137" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="D12" s="113">
         <f>D10/2048*1000</f>
         <v>0.12471466064453124</v>
       </c>
       <c r="E12" s="113" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
     </row>
     <row r="13" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C13" s="137" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="D13" s="113">
         <f>D11/2048*1000</f>
         <v>0.25187072753906248</v>
       </c>
       <c r="E13" s="113" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
     </row>
     <row r="14" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C14" s="137" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="D14" s="113">
         <f>INT(D12*1000/D3)-1</f>
@@ -19482,7 +19860,7 @@
     </row>
     <row r="15" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C15" s="137" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="D15" s="113">
         <f>D14</f>
@@ -19492,7 +19870,7 @@
     </row>
     <row r="16" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C16" s="137" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="D16" s="113">
         <f>INT(D13*1000/D3)-1</f>
@@ -19506,7 +19884,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63016306-17E7-4384-B0DF-AD6EB71951D7}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
@@ -19517,7 +19895,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D177CD4-6F93-4888-87F8-80C311E32BF1}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
@@ -19526,15 +19904,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D53A53DC-F305-461A-B42D-7174635AF376}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
-  <sheetData/>
-  <phoneticPr fontId="3" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>